<commit_message>
Add Total-exchange view alongside Sports view
- pullers (polymarket_us, cdna, rothera) now also emit all-category volume
- unified_sports_volume.py writes unified_sports_volume.csv (sports) +
  unified_total_volume.csv (whole exchange); Kalshi sports = single-leg + parlay
- make_excel.py: 4 tabs (Sports volume / Total exchange / Parlay share / Notes)
- dashboard + methodology updated
</commit_message>
<xml_diff>
--- a/unified_sports_volume.xlsx
+++ b/unified_sports_volume.xlsx
@@ -7,13 +7,15 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Daily volume" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Parlay share" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Notes" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Sports volume" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Total exchange" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Parlay share" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Notes" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Daily volume'!$A$2:$R$38</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Parlay share'!$A$2:$M$38</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Sports volume'!$A$2:$R$39</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Total exchange'!$A$2:$Q$39</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Parlay share'!$A$2:$M$39</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -45,7 +47,7 @@
     </font>
     <font>
       <b val="1"/>
-      <sz val="12"/>
+      <sz val="11"/>
     </font>
   </fonts>
   <fills count="5">
@@ -477,7 +479,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R38"/>
+  <dimension ref="A1:R39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -616,7 +618,7 @@
         </is>
       </c>
       <c r="B3" s="5" t="n">
-        <v>1410000000</v>
+        <v>1226348301.09</v>
       </c>
       <c r="C3" s="6" t="n">
         <v>133399888.66</v>
@@ -635,10 +637,10 @@
         <v>4370899</v>
       </c>
       <c r="I3" s="7" t="n">
-        <v>1587962094.58</v>
+        <v>1404310395.67</v>
       </c>
       <c r="J3" s="8" t="n">
-        <v>391416000</v>
+        <v>290712233.4</v>
       </c>
       <c r="K3" s="9" t="n">
         <v>50986272.22</v>
@@ -648,16 +650,16 @@
         <v>436176.76</v>
       </c>
       <c r="N3" s="9" t="n">
-        <v>597930.11</v>
+        <v>524812.1800000001</v>
       </c>
       <c r="O3" s="9" t="n">
-        <v>10664366.25</v>
+        <v>9360273.49</v>
       </c>
       <c r="P3" s="9" t="n">
         <v>2035457.65</v>
       </c>
       <c r="Q3" s="9" t="n">
-        <v>456136202.99</v>
+        <v>354055225.7</v>
       </c>
       <c r="R3" s="10" t="n">
         <v>0.08714584215412201</v>
@@ -670,7 +672,7 @@
         </is>
       </c>
       <c r="B4" s="5" t="n">
-        <v>1240000000</v>
+        <v>1019790521.49</v>
       </c>
       <c r="C4" s="6" t="n">
         <v>134065934.54</v>
@@ -689,10 +691,10 @@
         <v>7690938</v>
       </c>
       <c r="I4" s="7" t="n">
-        <v>1423404909.51</v>
+        <v>1203195431</v>
       </c>
       <c r="J4" s="8" t="n">
-        <v>344224000</v>
+        <v>223745816.63</v>
       </c>
       <c r="K4" s="9" t="n">
         <v>51144509.72</v>
@@ -702,16 +704,16 @@
         <v>484971.88</v>
       </c>
       <c r="N4" s="9" t="n">
-        <v>621319.9</v>
+        <v>516298.92</v>
       </c>
       <c r="O4" s="9" t="n">
-        <v>11116379.04</v>
+        <v>9237390.460000001</v>
       </c>
       <c r="P4" s="9" t="n">
         <v>3928624.18</v>
       </c>
       <c r="Q4" s="9" t="n">
-        <v>411519804.72</v>
+        <v>289057611.79</v>
       </c>
       <c r="R4" s="10" t="n">
         <v>0.07635377691307524</v>
@@ -724,7 +726,7 @@
         </is>
       </c>
       <c r="B5" s="5" t="n">
-        <v>826100000</v>
+        <v>766399762</v>
       </c>
       <c r="C5" s="6" t="n">
         <v>85344135.09999999</v>
@@ -743,10 +745,10 @@
         <v>9061437</v>
       </c>
       <c r="I5" s="7" t="n">
-        <v>942142547.04</v>
+        <v>882442309.04</v>
       </c>
       <c r="J5" s="8" t="n">
-        <v>229325360</v>
+        <v>197400001.9</v>
       </c>
       <c r="K5" s="9" t="n">
         <v>31777180.84</v>
@@ -756,16 +758,16 @@
         <v>165403.4</v>
       </c>
       <c r="N5" s="9" t="n">
-        <v>398283.4</v>
+        <v>374709.28</v>
       </c>
       <c r="O5" s="9" t="n">
-        <v>5739032.4</v>
+        <v>5399343.04</v>
       </c>
       <c r="P5" s="9" t="n">
         <v>4372698.14</v>
       </c>
       <c r="Q5" s="9" t="n">
-        <v>271777958.18</v>
+        <v>239489336.6</v>
       </c>
       <c r="R5" s="10" t="n">
         <v>0.05231046649197771</v>
@@ -778,7 +780,7 @@
         </is>
       </c>
       <c r="B6" s="5" t="n">
-        <v>1150000000</v>
+        <v>983748421.3200001</v>
       </c>
       <c r="C6" s="6" t="n">
         <v>120394335.41</v>
@@ -799,10 +801,10 @@
         <v>16424385</v>
       </c>
       <c r="I6" s="7" t="n">
-        <v>1334638149.02</v>
+        <v>1168386570.34</v>
       </c>
       <c r="J6" s="8" t="n">
-        <v>319240000</v>
+        <v>236058435.39</v>
       </c>
       <c r="K6" s="9" t="n">
         <v>47471997.74</v>
@@ -814,16 +816,16 @@
         <v>222905.14</v>
       </c>
       <c r="N6" s="9" t="n">
-        <v>362261.57</v>
+        <v>324586.19</v>
       </c>
       <c r="O6" s="9" t="n">
-        <v>8212604.46</v>
+        <v>7358489.61</v>
       </c>
       <c r="P6" s="9" t="n">
         <v>8062430.32</v>
       </c>
       <c r="Q6" s="9" t="n">
-        <v>389928450.59</v>
+        <v>305855095.76</v>
       </c>
       <c r="R6" s="10" t="n">
         <v>0.1040882840699126</v>
@@ -836,7 +838,7 @@
         </is>
       </c>
       <c r="B7" s="5" t="n">
-        <v>1300000000</v>
+        <v>1097580318.95</v>
       </c>
       <c r="C7" s="6" t="n">
         <v>125055737.8</v>
@@ -857,10 +859,10 @@
         <v>25367258</v>
       </c>
       <c r="I7" s="7" t="n">
-        <v>1505080037.58</v>
+        <v>1302660356.53</v>
       </c>
       <c r="J7" s="8" t="n">
-        <v>360880000</v>
+        <v>250948122.31</v>
       </c>
       <c r="K7" s="9" t="n">
         <v>47948549.82</v>
@@ -872,16 +874,16 @@
         <v>292548.17</v>
       </c>
       <c r="N7" s="9" t="n">
-        <v>822855.03</v>
+        <v>709925.6800000001</v>
       </c>
       <c r="O7" s="9" t="n">
-        <v>8917132.41</v>
+        <v>7693337.29</v>
       </c>
       <c r="P7" s="9" t="n">
         <v>12897725.83</v>
       </c>
       <c r="Q7" s="9" t="n">
-        <v>439320718.7</v>
+        <v>328052116.54</v>
       </c>
       <c r="R7" s="10" t="n">
         <v>0.1036604405692761</v>
@@ -894,7 +896,7 @@
         </is>
       </c>
       <c r="B8" s="5" t="n">
-        <v>1180000000</v>
+        <v>1011514178.87</v>
       </c>
       <c r="C8" s="6" t="n">
         <v>141146850.05</v>
@@ -915,10 +917,10 @@
         <v>23442413</v>
       </c>
       <c r="I8" s="7" t="n">
-        <v>1402173119.51</v>
+        <v>1233687298.38</v>
       </c>
       <c r="J8" s="8" t="n">
-        <v>327568000</v>
+        <v>229522489.57</v>
       </c>
       <c r="K8" s="9" t="n">
         <v>50551741.94</v>
@@ -930,16 +932,16 @@
         <v>314539.43</v>
       </c>
       <c r="N8" s="9" t="n">
-        <v>1460836.55</v>
+        <v>1255741.5</v>
       </c>
       <c r="O8" s="9" t="n">
-        <v>9783240.49</v>
+        <v>8409716.380000001</v>
       </c>
       <c r="P8" s="9" t="n">
         <v>11914017.45</v>
       </c>
       <c r="Q8" s="9" t="n">
-        <v>408821533.7</v>
+        <v>309197404.1</v>
       </c>
       <c r="R8" s="10" t="n">
         <v>0.09320593928966855</v>
@@ -952,7 +954,7 @@
         </is>
       </c>
       <c r="B9" s="5" t="n">
-        <v>1160000000</v>
+        <v>961933487.02</v>
       </c>
       <c r="C9" s="6" t="n">
         <v>117925601.54</v>
@@ -973,10 +975,10 @@
         <v>18014225</v>
       </c>
       <c r="I9" s="7" t="n">
-        <v>1343607161.54</v>
+        <v>1145540648.56</v>
       </c>
       <c r="J9" s="8" t="n">
-        <v>322016000</v>
+        <v>214888229.88</v>
       </c>
       <c r="K9" s="9" t="n">
         <v>44939973.52</v>
@@ -988,16 +990,16 @@
         <v>280061.26</v>
       </c>
       <c r="N9" s="9" t="n">
-        <v>962747.51</v>
+        <v>814778.05</v>
       </c>
       <c r="O9" s="9" t="n">
-        <v>8094646.96</v>
+        <v>6850540.39</v>
       </c>
       <c r="P9" s="9" t="n">
         <v>8768403.85</v>
       </c>
       <c r="Q9" s="9" t="n">
-        <v>389725239.67</v>
+        <v>281205393.52</v>
       </c>
       <c r="R9" s="10" t="n">
         <v>0.100308786205459</v>
@@ -1010,7 +1012,7 @@
         </is>
       </c>
       <c r="B10" s="5" t="n">
-        <v>1290000000</v>
+        <v>1073038713.76</v>
       </c>
       <c r="C10" s="6" t="n">
         <v>119094679.49</v>
@@ -1031,10 +1033,10 @@
         <v>23158725</v>
       </c>
       <c r="I10" s="7" t="n">
-        <v>1494665897.48</v>
+        <v>1277704611.24</v>
       </c>
       <c r="J10" s="8" t="n">
-        <v>358104000</v>
+        <v>240123237.17</v>
       </c>
       <c r="K10" s="9" t="n">
         <v>44015511.37</v>
@@ -1046,16 +1048,16 @@
         <v>545929.65</v>
       </c>
       <c r="N10" s="9" t="n">
-        <v>2779825.18</v>
+        <v>2353400.13</v>
       </c>
       <c r="O10" s="9" t="n">
-        <v>8941548.68</v>
+        <v>7569915.52</v>
       </c>
       <c r="P10" s="9" t="n">
         <v>11672366.2</v>
       </c>
       <c r="Q10" s="9" t="n">
-        <v>433525851.74</v>
+        <v>313747030.7</v>
       </c>
       <c r="R10" s="10" t="n">
         <v>0.1305164739611011</v>
@@ -1068,7 +1070,7 @@
         </is>
       </c>
       <c r="B11" s="5" t="n">
-        <v>1170000000</v>
+        <v>960754930.92</v>
       </c>
       <c r="C11" s="6" t="n">
         <v>126075255.12</v>
@@ -1089,10 +1091,10 @@
         <v>33913543</v>
       </c>
       <c r="I11" s="7" t="n">
-        <v>1394673317.12</v>
+        <v>1185428248.04</v>
       </c>
       <c r="J11" s="8" t="n">
-        <v>324792000</v>
+        <v>212543726.02</v>
       </c>
       <c r="K11" s="9" t="n">
         <v>48533344.05</v>
@@ -1104,16 +1106,16 @@
         <v>391311.2</v>
       </c>
       <c r="N11" s="9" t="n">
-        <v>2933210.13</v>
+        <v>2490144.51</v>
       </c>
       <c r="O11" s="9" t="n">
-        <v>10518020.08</v>
+        <v>8929257.99</v>
       </c>
       <c r="P11" s="9" t="n">
         <v>17131109.38</v>
       </c>
       <c r="Q11" s="9" t="n">
-        <v>410458570.91</v>
+        <v>296178469.23</v>
       </c>
       <c r="R11" s="10" t="n">
         <v>0.1174147553025735</v>
@@ -1126,7 +1128,7 @@
         </is>
       </c>
       <c r="B12" s="5" t="n">
-        <v>861600000</v>
+        <v>686488587.74</v>
       </c>
       <c r="C12" s="6" t="n">
         <v>76773291.01000001</v>
@@ -1147,10 +1149,10 @@
         <v>11323712</v>
       </c>
       <c r="I12" s="7" t="n">
-        <v>988511691.03</v>
+        <v>813400278.77</v>
       </c>
       <c r="J12" s="8" t="n">
-        <v>239180160</v>
+        <v>150986874.89</v>
       </c>
       <c r="K12" s="9" t="n">
         <v>28141958.88</v>
@@ -1162,16 +1164,16 @@
         <v>146839.93</v>
       </c>
       <c r="N12" s="9" t="n">
-        <v>2270938.56</v>
+        <v>1897060.47</v>
       </c>
       <c r="O12" s="9" t="n">
-        <v>4172455.9</v>
+        <v>3485519.72</v>
       </c>
       <c r="P12" s="9" t="n">
         <v>5809820.01</v>
       </c>
       <c r="Q12" s="9" t="n">
-        <v>285505514.36</v>
+        <v>196251414.98</v>
       </c>
       <c r="R12" s="10" t="n">
         <v>0.1320471995718654</v>
@@ -1184,7 +1186,7 @@
         </is>
       </c>
       <c r="B13" s="5" t="n">
-        <v>1180000000</v>
+        <v>970895177.89</v>
       </c>
       <c r="C13" s="6" t="n">
         <v>86060025.34</v>
@@ -1205,10 +1207,10 @@
         <v>19659153</v>
       </c>
       <c r="I13" s="7" t="n">
-        <v>1339556654.24</v>
+        <v>1130451832.13</v>
       </c>
       <c r="J13" s="8" t="n">
-        <v>327568000</v>
+        <v>227536176.85</v>
       </c>
       <c r="K13" s="9" t="n">
         <v>32573678.23</v>
@@ -1220,16 +1222,16 @@
         <v>342568.77</v>
       </c>
       <c r="N13" s="9" t="n">
-        <v>3016973.98</v>
+        <v>2642012.55</v>
       </c>
       <c r="O13" s="9" t="n">
-        <v>6295526.18</v>
+        <v>5513093.35</v>
       </c>
       <c r="P13" s="9" t="n">
         <v>9689300.880000001</v>
       </c>
       <c r="Q13" s="9" t="n">
-        <v>387723048.6</v>
+        <v>286533831.19</v>
       </c>
       <c r="R13" s="10" t="n">
         <v>0.1581581529884586</v>
@@ -1242,7 +1244,7 @@
         </is>
       </c>
       <c r="B14" s="5" t="n">
-        <v>1300000000</v>
+        <v>1042720983.61</v>
       </c>
       <c r="C14" s="6" t="n">
         <v>114182203.82</v>
@@ -1263,10 +1265,10 @@
         <v>23900271</v>
       </c>
       <c r="I14" s="7" t="n">
-        <v>1501484190.07</v>
+        <v>1244205173.68</v>
       </c>
       <c r="J14" s="8" t="n">
-        <v>360880000</v>
+        <v>230879117.13</v>
       </c>
       <c r="K14" s="9" t="n">
         <v>44020201.24</v>
@@ -1278,16 +1280,16 @@
         <v>463531.04</v>
       </c>
       <c r="N14" s="9" t="n">
-        <v>3398793</v>
+        <v>2865649.45</v>
       </c>
       <c r="O14" s="9" t="n">
-        <v>8333200.03</v>
+        <v>7026032.49</v>
       </c>
       <c r="P14" s="9" t="n">
         <v>11689925.33</v>
       </c>
       <c r="Q14" s="9" t="n">
-        <v>437525064.47</v>
+        <v>305683870.5</v>
       </c>
       <c r="R14" s="10" t="n">
         <v>0.1369006174109096</v>
@@ -1300,7 +1302,7 @@
         </is>
       </c>
       <c r="B15" s="5" t="n">
-        <v>1220000000</v>
+        <v>1046511668.87</v>
       </c>
       <c r="C15" s="6" t="n">
         <v>130618679.53</v>
@@ -1321,10 +1323,10 @@
         <v>24114127</v>
       </c>
       <c r="I15" s="7" t="n">
-        <v>1442047099.81</v>
+        <v>1268558768.68</v>
       </c>
       <c r="J15" s="8" t="n">
-        <v>338672000</v>
+        <v>238375725.51</v>
       </c>
       <c r="K15" s="9" t="n">
         <v>47519466.33</v>
@@ -1336,16 +1338,16 @@
         <v>401500.01</v>
       </c>
       <c r="N15" s="9" t="n">
-        <v>4351928.21</v>
+        <v>3737679.55</v>
       </c>
       <c r="O15" s="9" t="n">
-        <v>9126364.98</v>
+        <v>7838233.09</v>
       </c>
       <c r="P15" s="9" t="n">
         <v>11390787.92</v>
       </c>
       <c r="Q15" s="9" t="n">
-        <v>418041029.99</v>
+        <v>315842374.95</v>
       </c>
       <c r="R15" s="10" t="n">
         <v>0.1338434618903201</v>
@@ -1358,7 +1360,7 @@
         </is>
       </c>
       <c r="B16" s="5" t="n">
-        <v>1200000000</v>
+        <v>1026507894.75</v>
       </c>
       <c r="C16" s="6" t="n">
         <v>122512075.89</v>
@@ -1379,10 +1381,10 @@
         <v>13420824</v>
       </c>
       <c r="I16" s="7" t="n">
-        <v>1402143879.03</v>
+        <v>1228651773.78</v>
       </c>
       <c r="J16" s="8" t="n">
-        <v>333120000</v>
+        <v>246149823.25</v>
       </c>
       <c r="K16" s="9" t="n">
         <v>44967846.15</v>
@@ -1394,16 +1396,16 @@
         <v>598777.14</v>
       </c>
       <c r="N16" s="9" t="n">
-        <v>3991051.15</v>
+        <v>3558650.45</v>
       </c>
       <c r="O16" s="9" t="n">
-        <v>8453164.18</v>
+        <v>7537326.75</v>
       </c>
       <c r="P16" s="9" t="n">
         <v>5908662.92</v>
       </c>
       <c r="Q16" s="9" t="n">
-        <v>403888269.48</v>
+        <v>315569854.61</v>
       </c>
       <c r="R16" s="10" t="n">
         <v>0.1467243571212392</v>
@@ -1416,7 +1418,7 @@
         </is>
       </c>
       <c r="B17" s="5" t="n">
-        <v>1500000000</v>
+        <v>1275197725.87</v>
       </c>
       <c r="C17" s="6" t="n">
         <v>135215397.14</v>
@@ -1437,10 +1439,10 @@
         <v>23624339</v>
       </c>
       <c r="I17" s="7" t="n">
-        <v>1742721477.25</v>
+        <v>1517919203.12</v>
       </c>
       <c r="J17" s="8" t="n">
-        <v>416400000</v>
+        <v>295667968.4</v>
       </c>
       <c r="K17" s="9" t="n">
         <v>48968794.7</v>
@@ -1452,16 +1454,16 @@
         <v>899431.51</v>
       </c>
       <c r="N17" s="9" t="n">
-        <v>4926894.39</v>
+        <v>4271142.9</v>
       </c>
       <c r="O17" s="9" t="n">
-        <v>11052215.46</v>
+        <v>9581206.310000001</v>
       </c>
       <c r="P17" s="9" t="n">
         <v>11142968.25</v>
       </c>
       <c r="Q17" s="9" t="n">
-        <v>501623105.73</v>
+        <v>378764313.5</v>
       </c>
       <c r="R17" s="10" t="n">
         <v>0.1671310595982739</v>
@@ -1474,7 +1476,7 @@
         </is>
       </c>
       <c r="B18" s="5" t="n">
-        <v>1400000000</v>
+        <v>1123162110.77</v>
       </c>
       <c r="C18" s="6" t="n">
         <v>146617403.12</v>
@@ -1495,10 +1497,10 @@
         <v>24327302</v>
       </c>
       <c r="I18" s="7" t="n">
-        <v>1652175161.33</v>
+        <v>1375337272.1</v>
       </c>
       <c r="J18" s="8" t="n">
-        <v>388640000</v>
+        <v>251871816.77</v>
       </c>
       <c r="K18" s="9" t="n">
         <v>56978627.74</v>
@@ -1510,16 +1512,16 @@
         <v>644960.33</v>
       </c>
       <c r="N18" s="9" t="n">
-        <v>4127549.32</v>
+        <v>3520463.22</v>
       </c>
       <c r="O18" s="9" t="n">
-        <v>13196617.46</v>
+        <v>11255639.31</v>
       </c>
       <c r="P18" s="9" t="n">
         <v>11565704.7</v>
       </c>
       <c r="Q18" s="9" t="n">
-        <v>480407123.62</v>
+        <v>341090876.14</v>
       </c>
       <c r="R18" s="10" t="n">
         <v>0.1404248555660547</v>
@@ -1532,7 +1534,7 @@
         </is>
       </c>
       <c r="B19" s="5" t="n">
-        <v>926400000</v>
+        <v>780468036.02</v>
       </c>
       <c r="C19" s="6" t="n">
         <v>100434174.96</v>
@@ -1553,10 +1555,10 @@
         <v>11675481</v>
       </c>
       <c r="I19" s="7" t="n">
-        <v>1087816845.53</v>
+        <v>941884881.55</v>
       </c>
       <c r="J19" s="8" t="n">
-        <v>257168640</v>
+        <v>182876983.93</v>
       </c>
       <c r="K19" s="9" t="n">
         <v>36933011.94</v>
@@ -1568,16 +1570,16 @@
         <v>587784.12</v>
       </c>
       <c r="N19" s="9" t="n">
-        <v>3290649.79</v>
+        <v>2893225.33</v>
       </c>
       <c r="O19" s="9" t="n">
-        <v>5662876.63</v>
+        <v>4978949.19</v>
       </c>
       <c r="P19" s="9" t="n">
         <v>5508381.8</v>
       </c>
       <c r="Q19" s="9" t="n">
-        <v>315734009.35</v>
+        <v>240361001.38</v>
       </c>
       <c r="R19" s="10" t="n">
         <v>0.1248997633733931</v>
@@ -1590,7 +1592,7 @@
         </is>
       </c>
       <c r="B20" s="5" t="n">
-        <v>1160000000</v>
+        <v>925190752.63</v>
       </c>
       <c r="C20" s="6" t="n">
         <v>104121932.82</v>
@@ -1611,10 +1613,10 @@
         <v>14628870</v>
       </c>
       <c r="I20" s="7" t="n">
-        <v>1338003383.82</v>
+        <v>1103194136.45</v>
       </c>
       <c r="J20" s="8" t="n">
-        <v>322016000</v>
+        <v>208930058.54</v>
       </c>
       <c r="K20" s="9" t="n">
         <v>38002578.37</v>
@@ -1626,16 +1628,16 @@
         <v>262338.04</v>
       </c>
       <c r="N20" s="9" t="n">
-        <v>3637816.9</v>
+        <v>3099127.65</v>
       </c>
       <c r="O20" s="9" t="n">
-        <v>7299548.29</v>
+        <v>6218628.53</v>
       </c>
       <c r="P20" s="9" t="n">
         <v>6862320.27</v>
       </c>
       <c r="Q20" s="9" t="n">
-        <v>385453875.2</v>
+        <v>270748324.73</v>
       </c>
       <c r="R20" s="10" t="n">
         <v>0.178213812300984</v>
@@ -1648,7 +1650,7 @@
         </is>
       </c>
       <c r="B21" s="5" t="n">
-        <v>1370000000</v>
+        <v>1099235509.23</v>
       </c>
       <c r="C21" s="6" t="n">
         <v>122677612.96</v>
@@ -1669,10 +1671,10 @@
         <v>21296436</v>
       </c>
       <c r="I21" s="7" t="n">
-        <v>1585300293.82</v>
+        <v>1314535803.05</v>
       </c>
       <c r="J21" s="8" t="n">
-        <v>380312000</v>
+        <v>244612818.63</v>
       </c>
       <c r="K21" s="9" t="n">
         <v>44708007.56</v>
@@ -1684,16 +1686,16 @@
         <v>691813.04</v>
       </c>
       <c r="N21" s="9" t="n">
-        <v>4357451.88</v>
+        <v>3671151</v>
       </c>
       <c r="O21" s="9" t="n">
-        <v>9151899.65</v>
+        <v>7710470.83</v>
       </c>
       <c r="P21" s="9" t="n">
         <v>10373288.39</v>
       </c>
       <c r="Q21" s="9" t="n">
-        <v>457293772.23</v>
+        <v>319466861.16</v>
       </c>
       <c r="R21" s="10" t="n">
         <v>0.2003579150386557</v>
@@ -1706,7 +1708,7 @@
         </is>
       </c>
       <c r="B22" s="5" t="n">
-        <v>1190000000</v>
+        <v>967567863.75</v>
       </c>
       <c r="C22" s="6" t="n">
         <v>132905659.86</v>
@@ -1727,10 +1729,10 @@
         <v>24665675</v>
       </c>
       <c r="I22" s="7" t="n">
-        <v>1413321005.58</v>
+        <v>1190888869.33</v>
       </c>
       <c r="J22" s="8" t="n">
-        <v>330344000</v>
+        <v>210526920.69</v>
       </c>
       <c r="K22" s="9" t="n">
         <v>44439935.08</v>
@@ -1742,16 +1744,16 @@
         <v>426029.96</v>
       </c>
       <c r="N22" s="9" t="n">
-        <v>3954335.84</v>
+        <v>3281796.18</v>
       </c>
       <c r="O22" s="9" t="n">
-        <v>9080706.52</v>
+        <v>7536291.6</v>
       </c>
       <c r="P22" s="9" t="n">
         <v>11601612.35</v>
       </c>
       <c r="Q22" s="9" t="n">
-        <v>405843923.03</v>
+        <v>283809889.14</v>
       </c>
       <c r="R22" s="10" t="n">
         <v>0.180964978836361</v>
@@ -1764,7 +1766,7 @@
         </is>
       </c>
       <c r="B23" s="5" t="n">
-        <v>1260000000</v>
+        <v>1003048142.35</v>
       </c>
       <c r="C23" s="6" t="n">
         <v>118302722.67</v>
@@ -1785,10 +1787,10 @@
         <v>9456461</v>
       </c>
       <c r="I23" s="7" t="n">
-        <v>1455156688.06</v>
+        <v>1198204830.41</v>
       </c>
       <c r="J23" s="8" t="n">
-        <v>349776000</v>
+        <v>222078381.47</v>
       </c>
       <c r="K23" s="9" t="n">
         <v>35142057.4</v>
@@ -1800,16 +1802,16 @@
         <v>577229.27</v>
       </c>
       <c r="N23" s="9" t="n">
-        <v>4683619.92</v>
+        <v>3890999.55</v>
       </c>
       <c r="O23" s="9" t="n">
-        <v>7626528.18</v>
+        <v>6335872.31</v>
       </c>
       <c r="P23" s="9" t="n">
         <v>3594255.85</v>
       </c>
       <c r="Q23" s="9" t="n">
-        <v>410790643.03</v>
+        <v>281009748.26</v>
       </c>
       <c r="R23" s="10" t="n">
         <v>0.316619068118602</v>
@@ -1822,7 +1824,7 @@
         </is>
       </c>
       <c r="B24" s="5" t="n">
-        <v>1680000000</v>
+        <v>1362246646.22</v>
       </c>
       <c r="C24" s="6" t="n">
         <v>146513108.49</v>
@@ -1843,10 +1845,10 @@
         <v>21014051</v>
       </c>
       <c r="I24" s="7" t="n">
-        <v>1952216755.12</v>
+        <v>1634463401.34</v>
       </c>
       <c r="J24" s="8" t="n">
-        <v>466368000</v>
+        <v>306752950.06</v>
       </c>
       <c r="K24" s="9" t="n">
         <v>43271898.85</v>
@@ -1858,16 +1860,16 @@
         <v>545961.96</v>
       </c>
       <c r="N24" s="9" t="n">
-        <v>7292030.85</v>
+        <v>6136465.49</v>
       </c>
       <c r="O24" s="9" t="n">
-        <v>12204614.9</v>
+        <v>10270554.21</v>
       </c>
       <c r="P24" s="9" t="n">
         <v>9618578.710000001</v>
       </c>
       <c r="Q24" s="9" t="n">
-        <v>550716777.25</v>
+        <v>388012101.25</v>
       </c>
       <c r="R24" s="10" t="n">
         <v>0.3069045894333504</v>
@@ -1880,7 +1882,7 @@
         </is>
       </c>
       <c r="B25" s="5" t="n">
-        <v>1480000000</v>
+        <v>1156848829.83</v>
       </c>
       <c r="C25" s="6" t="n">
         <v>144797057.56</v>
@@ -1901,10 +1903,10 @@
         <v>21174047</v>
       </c>
       <c r="I25" s="7" t="n">
-        <v>1732499967.65</v>
+        <v>1409348797.48</v>
       </c>
       <c r="J25" s="8" t="n">
-        <v>410848000</v>
+        <v>247783486.21</v>
       </c>
       <c r="K25" s="9" t="n">
         <v>45249277.15</v>
@@ -1916,16 +1918,16 @@
         <v>678289.72</v>
       </c>
       <c r="N25" s="9" t="n">
-        <v>4661314.97</v>
+        <v>3795191.26</v>
       </c>
       <c r="O25" s="9" t="n">
-        <v>12195295.41</v>
+        <v>9929275.09</v>
       </c>
       <c r="P25" s="9" t="n">
         <v>10104181.45</v>
       </c>
       <c r="Q25" s="9" t="n">
-        <v>492177835.15</v>
+        <v>325981177.34</v>
       </c>
       <c r="R25" s="10" t="n">
         <v>0.2790295913221863</v>
@@ -1938,7 +1940,7 @@
         </is>
       </c>
       <c r="B26" s="5" t="n">
-        <v>1120000000</v>
+        <v>870234303.1799999</v>
       </c>
       <c r="C26" s="6" t="n">
         <v>97537800.47</v>
@@ -1959,10 +1961,10 @@
         <v>11503296</v>
       </c>
       <c r="I26" s="7" t="n">
-        <v>1289104212.37</v>
+        <v>1039338515.55</v>
       </c>
       <c r="J26" s="8" t="n">
-        <v>310912000</v>
+        <v>193417623.28</v>
       </c>
       <c r="K26" s="9" t="n">
         <v>31464287.45</v>
@@ -1974,16 +1976,16 @@
         <v>240533.84</v>
       </c>
       <c r="N26" s="9" t="n">
-        <v>3901805.72</v>
+        <v>3256064.62</v>
       </c>
       <c r="O26" s="9" t="n">
-        <v>6811497.3</v>
+        <v>5684208.02</v>
       </c>
       <c r="P26" s="9" t="n">
         <v>5132563.13</v>
       </c>
       <c r="Q26" s="9" t="n">
-        <v>364527114.66</v>
+        <v>245259707.55</v>
       </c>
       <c r="R26" s="10" t="n">
         <v>0.2509415863550032</v>
@@ -1996,7 +1998,7 @@
         </is>
       </c>
       <c r="B27" s="5" t="n">
-        <v>1320000000</v>
+        <v>1002162415.6</v>
       </c>
       <c r="C27" s="6" t="n">
         <v>122103455.85</v>
@@ -2017,10 +2019,10 @@
         <v>16332836</v>
       </c>
       <c r="I27" s="7" t="n">
-        <v>1527337407.96</v>
+        <v>1209499823.56</v>
       </c>
       <c r="J27" s="8" t="n">
-        <v>366432000</v>
+        <v>216979327.6</v>
       </c>
       <c r="K27" s="9" t="n">
         <v>38650744.49</v>
@@ -2032,16 +2034,16 @@
         <v>345067.73</v>
       </c>
       <c r="N27" s="9" t="n">
-        <v>3577500.59</v>
+        <v>2934170.27</v>
       </c>
       <c r="O27" s="9" t="n">
-        <v>8458913.27</v>
+        <v>6937774.34</v>
       </c>
       <c r="P27" s="9" t="n">
         <v>7469897.21</v>
       </c>
       <c r="Q27" s="9" t="n">
-        <v>432568818.94</v>
+        <v>280951677.29</v>
       </c>
       <c r="R27" s="10" t="n">
         <v>0.2836514946154119</v>
@@ -2054,7 +2056,7 @@
         </is>
       </c>
       <c r="B28" s="5" t="n">
-        <v>1420000000</v>
+        <v>1105872460</v>
       </c>
       <c r="C28" s="6" t="n">
         <v>146265225.05</v>
@@ -2075,10 +2077,10 @@
         <v>22808657</v>
       </c>
       <c r="I28" s="7" t="n">
-        <v>1665854899.65</v>
+        <v>1351727359.65</v>
       </c>
       <c r="J28" s="8" t="n">
-        <v>394192000</v>
+        <v>242452076.24</v>
       </c>
       <c r="K28" s="9" t="n">
         <v>47820263.66</v>
@@ -2090,16 +2092,16 @@
         <v>1170559.87</v>
       </c>
       <c r="N28" s="9" t="n">
-        <v>3228105.93</v>
+        <v>2693171.11</v>
       </c>
       <c r="O28" s="9" t="n">
-        <v>10504510.02</v>
+        <v>8763790.130000001</v>
       </c>
       <c r="P28" s="9" t="n">
         <v>10604681.86</v>
       </c>
       <c r="Q28" s="9" t="n">
-        <v>476781094.95</v>
+        <v>322765516.48</v>
       </c>
       <c r="R28" s="10" t="n">
         <v>0.2603327878455701</v>
@@ -2112,7 +2114,7 @@
         </is>
       </c>
       <c r="B29" s="5" t="n">
-        <v>1190000000</v>
+        <v>932777126.6900001</v>
       </c>
       <c r="C29" s="6" t="n">
         <v>110832888.3</v>
@@ -2133,10 +2135,10 @@
         <v>22948569</v>
       </c>
       <c r="I29" s="7" t="n">
-        <v>1393947814.45</v>
+        <v>1136724941.14</v>
       </c>
       <c r="J29" s="8" t="n">
-        <v>330344000</v>
+        <v>196501497.97</v>
       </c>
       <c r="K29" s="9" t="n">
         <v>33469362.8</v>
@@ -2148,16 +2150,16 @@
         <v>3504492.28</v>
       </c>
       <c r="N29" s="9" t="n">
-        <v>3640510.96</v>
+        <v>2927838.11</v>
       </c>
       <c r="O29" s="9" t="n">
-        <v>8178728.19</v>
+        <v>6577645.92</v>
       </c>
       <c r="P29" s="9" t="n">
         <v>9864047.33</v>
       </c>
       <c r="Q29" s="9" t="n">
-        <v>395611580.51</v>
+        <v>259455323.36</v>
       </c>
       <c r="R29" s="10" t="n">
         <v>0.2711837542671093</v>
@@ -2170,7 +2172,7 @@
         </is>
       </c>
       <c r="B30" s="5" t="n">
-        <v>1490000000</v>
+        <v>1161937950.78</v>
       </c>
       <c r="C30" s="6" t="n">
         <v>97591814.65000001</v>
@@ -2191,10 +2193,10 @@
         <v>14181446</v>
       </c>
       <c r="I30" s="7" t="n">
-        <v>1682836484.07</v>
+        <v>1354774434.85</v>
       </c>
       <c r="J30" s="8" t="n">
-        <v>413624000</v>
+        <v>252320947.82</v>
       </c>
       <c r="K30" s="9" t="n">
         <v>30161405.65</v>
@@ -2206,16 +2208,16 @@
         <v>5547393.25</v>
       </c>
       <c r="N30" s="9" t="n">
-        <v>5186852.71</v>
+        <v>4229055.32</v>
       </c>
       <c r="O30" s="9" t="n">
-        <v>5570098.34</v>
+        <v>4541531.32</v>
       </c>
       <c r="P30" s="9" t="n">
         <v>5642292.92</v>
       </c>
       <c r="Q30" s="9" t="n">
-        <v>475222669.68</v>
+        <v>311933253.09</v>
       </c>
       <c r="R30" s="10" t="n">
         <v>0.3089090135319407</v>
@@ -2228,7 +2230,7 @@
         </is>
       </c>
       <c r="B31" s="5" t="n">
-        <v>1930000000</v>
+        <v>1439894997.32</v>
       </c>
       <c r="C31" s="6" t="n">
         <v>164444551.54</v>
@@ -2249,10 +2251,10 @@
         <v>25879178</v>
       </c>
       <c r="I31" s="7" t="n">
-        <v>2230056666.03</v>
+        <v>1739951663.35</v>
       </c>
       <c r="J31" s="8" t="n">
-        <v>535768000</v>
+        <v>284684023.21</v>
       </c>
       <c r="K31" s="9" t="n">
         <v>46737225.01</v>
@@ -2264,16 +2266,16 @@
         <v>10477277.08</v>
       </c>
       <c r="N31" s="9" t="n">
-        <v>5320793.3</v>
+        <v>4066960.53</v>
       </c>
       <c r="O31" s="9" t="n">
-        <v>7821426.22</v>
+        <v>5978325.02</v>
       </c>
       <c r="P31" s="9" t="n">
         <v>11977848.09</v>
       </c>
       <c r="Q31" s="9" t="n">
-        <v>629735408.38</v>
+        <v>375554497.62</v>
       </c>
       <c r="R31" s="10" t="n">
         <v>0.3202852257171364</v>
@@ -2286,7 +2288,7 @@
         </is>
       </c>
       <c r="B32" s="5" t="n">
-        <v>1700000000</v>
+        <v>1319471126.18</v>
       </c>
       <c r="C32" s="6" t="n">
         <v>152797571.95</v>
@@ -2307,10 +2309,10 @@
         <v>30594436</v>
       </c>
       <c r="I32" s="7" t="n">
-        <v>1959763084.12</v>
+        <v>1579234210.3</v>
       </c>
       <c r="J32" s="8" t="n">
-        <v>471920000</v>
+        <v>283287864.82</v>
       </c>
       <c r="K32" s="9" t="n">
         <v>45961937.88</v>
@@ -2322,16 +2324,16 @@
         <v>1721674.99</v>
       </c>
       <c r="N32" s="9" t="n">
-        <v>3750230.46</v>
+        <v>3050704.66</v>
       </c>
       <c r="O32" s="9" t="n">
-        <v>9143248.68</v>
+        <v>7437769.93</v>
       </c>
       <c r="P32" s="9" t="n">
         <v>14143642.2</v>
       </c>
       <c r="Q32" s="9" t="n">
-        <v>554564843.66</v>
+        <v>363527703.93</v>
       </c>
       <c r="R32" s="10" t="n">
         <v>0.3068596818867773</v>
@@ -2344,7 +2346,7 @@
         </is>
       </c>
       <c r="B33" s="5" t="n">
-        <v>1400000000</v>
+        <v>1096650095.4</v>
       </c>
       <c r="C33" s="6" t="n">
         <v>112904481.21</v>
@@ -2365,10 +2367,10 @@
         <v>10653135</v>
       </c>
       <c r="I33" s="7" t="n">
-        <v>1586041026.11</v>
+        <v>1282691121.51</v>
       </c>
       <c r="J33" s="8" t="n">
-        <v>388640000</v>
+        <v>243300304.72</v>
       </c>
       <c r="K33" s="9" t="n">
         <v>36710222.03</v>
@@ -2380,16 +2382,16 @@
         <v>7580.34</v>
       </c>
       <c r="N33" s="9" t="n">
-        <v>1996993.35</v>
+        <v>1660372.72</v>
       </c>
       <c r="O33" s="9" t="n">
-        <v>8660854.789999999</v>
+        <v>7200948.89</v>
       </c>
       <c r="P33" s="9" t="n">
         <v>4972134.8</v>
       </c>
       <c r="Q33" s="9" t="n">
-        <v>449152739.67</v>
+        <v>302016517.86</v>
       </c>
       <c r="R33" s="10" t="n">
         <v>0.2945849325840212</v>
@@ -2402,7 +2404,7 @@
         </is>
       </c>
       <c r="B34" s="5" t="n">
-        <v>1520000000</v>
+        <v>1141713194.51</v>
       </c>
       <c r="C34" s="6" t="n">
         <v>111143033.33</v>
@@ -2423,10 +2425,10 @@
         <v>17975675</v>
       </c>
       <c r="I34" s="7" t="n">
-        <v>1743891113.95</v>
+        <v>1365604308.46</v>
       </c>
       <c r="J34" s="8" t="n">
-        <v>421952000</v>
+        <v>239505889.8</v>
       </c>
       <c r="K34" s="9" t="n">
         <v>33583851.03</v>
@@ -2438,16 +2440,16 @@
         <v>7000711.88</v>
       </c>
       <c r="N34" s="9" t="n">
-        <v>1629086.86</v>
+        <v>1298241.07</v>
       </c>
       <c r="O34" s="9" t="n">
-        <v>11585152.88</v>
+        <v>9232363.02</v>
       </c>
       <c r="P34" s="9" t="n">
         <v>8253527.4</v>
       </c>
       <c r="Q34" s="9" t="n">
-        <v>492426614.48</v>
+        <v>307296868.64</v>
       </c>
       <c r="R34" s="10" t="n">
         <v>0.3414174721986673</v>
@@ -2460,7 +2462,7 @@
         </is>
       </c>
       <c r="B35" s="5" t="n">
-        <v>1580000000</v>
+        <v>1192398704.86</v>
       </c>
       <c r="C35" s="6" t="n">
         <v>132482292.68</v>
@@ -2481,10 +2483,10 @@
         <v>24222748</v>
       </c>
       <c r="I35" s="7" t="n">
-        <v>1823657006.67</v>
+        <v>1436055711.53</v>
       </c>
       <c r="J35" s="8" t="n">
-        <v>438608000</v>
+        <v>253455797.87</v>
       </c>
       <c r="K35" s="9" t="n">
         <v>39009606.34</v>
@@ -2496,16 +2498,16 @@
         <v>7686788.4</v>
       </c>
       <c r="N35" s="9" t="n">
-        <v>2653790.16</v>
+        <v>2144828.4</v>
       </c>
       <c r="O35" s="9" t="n">
-        <v>8343840.94</v>
+        <v>6743602.9</v>
       </c>
       <c r="P35" s="9" t="n">
         <v>11819801.92</v>
       </c>
       <c r="Q35" s="9" t="n">
-        <v>515070033.3</v>
+        <v>327808631.37</v>
       </c>
       <c r="R35" s="10" t="n">
         <v>0.3444918139984984</v>
@@ -2518,7 +2520,7 @@
         </is>
       </c>
       <c r="B36" s="5" t="n">
-        <v>1540000000</v>
+        <v>1226269672.23</v>
       </c>
       <c r="C36" s="6" t="n">
         <v>147816672.25</v>
@@ -2539,10 +2541,10 @@
         <v>27056266</v>
       </c>
       <c r="I36" s="7" t="n">
-        <v>1807340290.87</v>
+        <v>1493609963.1</v>
       </c>
       <c r="J36" s="8" t="n">
-        <v>427504000</v>
+        <v>272681676.9</v>
       </c>
       <c r="K36" s="9" t="n">
         <v>47162206.4</v>
@@ -2554,16 +2556,16 @@
         <v>8799940.630000001</v>
       </c>
       <c r="N36" s="9" t="n">
-        <v>2975679.03</v>
+        <v>2511016.2</v>
       </c>
       <c r="O36" s="9" t="n">
-        <v>8586780.689999999</v>
+        <v>7245924.46</v>
       </c>
       <c r="P36" s="9" t="n">
         <v>13258351.53</v>
       </c>
       <c r="Q36" s="9" t="n">
-        <v>517548544.4</v>
+        <v>360920702.24</v>
       </c>
       <c r="R36" s="10" t="n">
         <v>0.3000842795719814</v>
@@ -2576,7 +2578,7 @@
         </is>
       </c>
       <c r="B37" s="5" t="n">
-        <v>1721050019.04</v>
+        <v>1172274619.91</v>
       </c>
       <c r="C37" s="6" t="n">
         <v>161563894</v>
@@ -2597,10 +2599,10 @@
         <v>12713214</v>
       </c>
       <c r="I37" s="7" t="n">
-        <v>1995370163.79</v>
+        <v>1446594764.66</v>
       </c>
       <c r="J37" s="8" t="n">
-        <v>477763485.29</v>
+        <v>244007566.85</v>
       </c>
       <c r="K37" s="9" t="n">
         <v>49969403.31</v>
@@ -2612,16 +2614,16 @@
         <v>7004156.33</v>
       </c>
       <c r="N37" s="9" t="n">
-        <v>2925215.83</v>
+        <v>2343656.88</v>
       </c>
       <c r="O37" s="9" t="n">
-        <v>10253660.7</v>
+        <v>8215141.66</v>
       </c>
       <c r="P37" s="9" t="n">
         <v>5644731.29</v>
       </c>
       <c r="Q37" s="9" t="n">
-        <v>563933268.61</v>
+        <v>327557272.18</v>
       </c>
       <c r="R37" s="10" t="n">
         <v>0.3158320960096582</v>
@@ -2633,9 +2635,7 @@
           <t>2026-09-05</t>
         </is>
       </c>
-      <c r="B38" s="5" t="n">
-        <v>2342612096.54</v>
-      </c>
+      <c r="B38" s="5" t="n"/>
       <c r="C38" s="6" t="n">
         <v>172439695.17</v>
       </c>
@@ -2655,11 +2655,9 @@
         <v>20531449</v>
       </c>
       <c r="I38" s="7" t="n">
-        <v>2686675158.6</v>
-      </c>
-      <c r="J38" s="8" t="n">
-        <v>650309118</v>
-      </c>
+        <v>344063062.06</v>
+      </c>
+      <c r="J38" s="8" t="n"/>
       <c r="K38" s="9" t="n">
         <v>46814559.69</v>
       </c>
@@ -2670,23 +2668,77 @@
         <v>15883449.41</v>
       </c>
       <c r="N38" s="9" t="n">
-        <v>5016245.58</v>
+        <v>5461948.41</v>
       </c>
       <c r="O38" s="9" t="n">
-        <v>8508038.390000001</v>
+        <v>9263993.560000001</v>
       </c>
       <c r="P38" s="9" t="n">
         <v>9731632.92</v>
       </c>
       <c r="Q38" s="9" t="n">
-        <v>754286169.73</v>
+        <v>105178709.74</v>
       </c>
       <c r="R38" s="10" t="n">
         <v>0.3730201375328469</v>
       </c>
     </row>
+    <row r="39">
+      <c r="A39" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="B39" s="5" t="n"/>
+      <c r="C39" s="6" t="n">
+        <v>131412975.25</v>
+      </c>
+      <c r="D39" s="6" t="n">
+        <v>32056055.97</v>
+      </c>
+      <c r="E39" s="6" t="n">
+        <v>35925674</v>
+      </c>
+      <c r="F39" s="6" t="n">
+        <v>21673332.38</v>
+      </c>
+      <c r="G39" s="6" t="n">
+        <v>32407752</v>
+      </c>
+      <c r="H39" s="6" t="n">
+        <v>33293997</v>
+      </c>
+      <c r="I39" s="7" t="n">
+        <v>286769786.6</v>
+      </c>
+      <c r="J39" s="8" t="n"/>
+      <c r="K39" s="9" t="n">
+        <v>38038258.86</v>
+      </c>
+      <c r="L39" s="9" t="n">
+        <v>13010644.31</v>
+      </c>
+      <c r="M39" s="9" t="n">
+        <v>11501420.69</v>
+      </c>
+      <c r="N39" s="9" t="n">
+        <v>7323631.12</v>
+      </c>
+      <c r="O39" s="9" t="n">
+        <v>10950896.56</v>
+      </c>
+      <c r="P39" s="9" t="n">
+        <v>16077465.82</v>
+      </c>
+      <c r="Q39" s="9" t="n">
+        <v>96902317.34999999</v>
+      </c>
+      <c r="R39" s="10" t="n">
+        <v>0.3654745795652588</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A2:R38"/>
+  <autoFilter ref="A2:R39"/>
   <mergeCells count="3">
     <mergeCell ref="R1"/>
     <mergeCell ref="B1:I1"/>
@@ -2702,7 +2754,2159 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M40"/>
+  <dimension ref="A1:Q39"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="8" max="8"/>
+    <col width="14" customWidth="1" min="9" max="9"/>
+    <col width="14" customWidth="1" min="10" max="10"/>
+    <col width="14" customWidth="1" min="11" max="11"/>
+    <col width="14" customWidth="1" min="12" max="12"/>
+    <col width="14" customWidth="1" min="13" max="13"/>
+    <col width="14" customWidth="1" min="14" max="14"/>
+    <col width="14" customWidth="1" min="15" max="15"/>
+    <col width="14" customWidth="1" min="16" max="16"/>
+    <col width="14" customWidth="1" min="17" max="17"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Contracts traded  (one-sided, $1 face)</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Notional $  (~ USD changed hands)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="B2" s="3" t="inlineStr">
+        <is>
+          <t>Kalshi</t>
+        </is>
+      </c>
+      <c r="C2" s="3" t="inlineStr">
+        <is>
+          <t>Polymarket US</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="inlineStr">
+        <is>
+          <t>Novig</t>
+        </is>
+      </c>
+      <c r="E2" s="3" t="inlineStr">
+        <is>
+          <t>DKeX</t>
+        </is>
+      </c>
+      <c r="F2" s="3" t="inlineStr">
+        <is>
+          <t>UDX</t>
+        </is>
+      </c>
+      <c r="G2" s="3" t="inlineStr">
+        <is>
+          <t>Crypto.com</t>
+        </is>
+      </c>
+      <c r="H2" s="3" t="inlineStr">
+        <is>
+          <t>Rothera</t>
+        </is>
+      </c>
+      <c r="I2" s="3" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+      <c r="J2" s="3" t="inlineStr">
+        <is>
+          <t>Kalshi</t>
+        </is>
+      </c>
+      <c r="K2" s="3" t="inlineStr">
+        <is>
+          <t>Polymarket US</t>
+        </is>
+      </c>
+      <c r="L2" s="3" t="inlineStr">
+        <is>
+          <t>Novig</t>
+        </is>
+      </c>
+      <c r="M2" s="3" t="inlineStr">
+        <is>
+          <t>DKeX</t>
+        </is>
+      </c>
+      <c r="N2" s="3" t="inlineStr">
+        <is>
+          <t>UDX</t>
+        </is>
+      </c>
+      <c r="O2" s="3" t="inlineStr">
+        <is>
+          <t>Crypto.com</t>
+        </is>
+      </c>
+      <c r="P2" s="3" t="inlineStr">
+        <is>
+          <t>Rothera</t>
+        </is>
+      </c>
+      <c r="Q2" s="3" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="4" t="inlineStr">
+        <is>
+          <t>2026-08-01</t>
+        </is>
+      </c>
+      <c r="B3" s="5" t="n">
+        <v>1410000000</v>
+      </c>
+      <c r="C3" s="6" t="n">
+        <v>134802912.52</v>
+      </c>
+      <c r="D3" s="6" t="n"/>
+      <c r="E3" s="6" t="n">
+        <v>983501</v>
+      </c>
+      <c r="F3" s="6" t="n">
+        <v>2081593.92</v>
+      </c>
+      <c r="G3" s="6" t="n">
+        <v>37483644</v>
+      </c>
+      <c r="H3" s="6" t="n">
+        <v>4563661</v>
+      </c>
+      <c r="I3" s="7" t="n">
+        <v>1589915312.44</v>
+      </c>
+      <c r="J3" s="8" t="n">
+        <v>391416000</v>
+      </c>
+      <c r="K3" s="9" t="n">
+        <v>51252892</v>
+      </c>
+      <c r="L3" s="9" t="n"/>
+      <c r="M3" s="9" t="n">
+        <v>436176.76</v>
+      </c>
+      <c r="N3" s="9" t="n">
+        <v>597732.41</v>
+      </c>
+      <c r="O3" s="9" t="n">
+        <v>10763477.26</v>
+      </c>
+      <c r="P3" s="9" t="n">
+        <v>2079977.15</v>
+      </c>
+      <c r="Q3" s="9" t="n">
+        <v>456546255.58</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>2026-08-02</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="n">
+        <v>1240000000</v>
+      </c>
+      <c r="C4" s="6" t="n">
+        <v>135833286.22</v>
+      </c>
+      <c r="D4" s="6" t="n"/>
+      <c r="E4" s="6" t="n">
+        <v>1048537</v>
+      </c>
+      <c r="F4" s="6" t="n">
+        <v>2149081.97</v>
+      </c>
+      <c r="G4" s="6" t="n">
+        <v>38952253</v>
+      </c>
+      <c r="H4" s="6" t="n">
+        <v>7899184</v>
+      </c>
+      <c r="I4" s="7" t="n">
+        <v>1425882342.19</v>
+      </c>
+      <c r="J4" s="8" t="n">
+        <v>344224000</v>
+      </c>
+      <c r="K4" s="9" t="n">
+        <v>51599931.62</v>
+      </c>
+      <c r="L4" s="9" t="n"/>
+      <c r="M4" s="9" t="n">
+        <v>484971.88</v>
+      </c>
+      <c r="N4" s="9" t="n">
+        <v>621241.21</v>
+      </c>
+      <c r="O4" s="9" t="n">
+        <v>11260037.98</v>
+      </c>
+      <c r="P4" s="9" t="n">
+        <v>3993660.15</v>
+      </c>
+      <c r="Q4" s="9" t="n">
+        <v>412183842.84</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="n">
+        <v>826100000</v>
+      </c>
+      <c r="C5" s="6" t="n">
+        <v>87736455.39</v>
+      </c>
+      <c r="D5" s="6" t="n"/>
+      <c r="E5" s="6" t="n">
+        <v>361422</v>
+      </c>
+      <c r="F5" s="6" t="n">
+        <v>1380684.94</v>
+      </c>
+      <c r="G5" s="6" t="n">
+        <v>20405362</v>
+      </c>
+      <c r="H5" s="6" t="n">
+        <v>9274058</v>
+      </c>
+      <c r="I5" s="7" t="n">
+        <v>945257982.33</v>
+      </c>
+      <c r="J5" s="8" t="n">
+        <v>229325360</v>
+      </c>
+      <c r="K5" s="9" t="n">
+        <v>32367279.06</v>
+      </c>
+      <c r="L5" s="9" t="n"/>
+      <c r="M5" s="9" t="n">
+        <v>165403.4</v>
+      </c>
+      <c r="N5" s="9" t="n">
+        <v>398141.79</v>
+      </c>
+      <c r="O5" s="9" t="n">
+        <v>5884200.74</v>
+      </c>
+      <c r="P5" s="9" t="n">
+        <v>4439328.3</v>
+      </c>
+      <c r="Q5" s="9" t="n">
+        <v>272579713.29</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="n">
+        <v>1150000000</v>
+      </c>
+      <c r="C6" s="6" t="n">
+        <v>122647218.83</v>
+      </c>
+      <c r="D6" s="6" t="n">
+        <v>17996650.04</v>
+      </c>
+      <c r="E6" s="6" t="n">
+        <v>472924</v>
+      </c>
+      <c r="F6" s="6" t="n">
+        <v>1239940.57</v>
+      </c>
+      <c r="G6" s="6" t="n">
+        <v>28486561</v>
+      </c>
+      <c r="H6" s="6" t="n">
+        <v>16628972</v>
+      </c>
+      <c r="I6" s="7" t="n">
+        <v>1337472266.44</v>
+      </c>
+      <c r="J6" s="8" t="n">
+        <v>319240000</v>
+      </c>
+      <c r="K6" s="9" t="n">
+        <v>48161416.36</v>
+      </c>
+      <c r="L6" s="9" t="n">
+        <v>6356251.37</v>
+      </c>
+      <c r="M6" s="9" t="n">
+        <v>222905.14</v>
+      </c>
+      <c r="N6" s="9" t="n">
+        <v>362287.47</v>
+      </c>
+      <c r="O6" s="9" t="n">
+        <v>8323241.01</v>
+      </c>
+      <c r="P6" s="9" t="n">
+        <v>8118311.67</v>
+      </c>
+      <c r="Q6" s="9" t="n">
+        <v>390784413.02</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>2026-08-05</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="n">
+        <v>1300000000</v>
+      </c>
+      <c r="C7" s="6" t="n">
+        <v>127635575.93</v>
+      </c>
+      <c r="D7" s="6" t="n">
+        <v>20682990.79</v>
+      </c>
+      <c r="E7" s="6" t="n">
+        <v>605580</v>
+      </c>
+      <c r="F7" s="6" t="n">
+        <v>2819039.99</v>
+      </c>
+      <c r="G7" s="6" t="n">
+        <v>30864670</v>
+      </c>
+      <c r="H7" s="6" t="n">
+        <v>25854868</v>
+      </c>
+      <c r="I7" s="7" t="n">
+        <v>1508462724.71</v>
+      </c>
+      <c r="J7" s="8" t="n">
+        <v>360880000</v>
+      </c>
+      <c r="K7" s="9" t="n">
+        <v>48492980.6</v>
+      </c>
+      <c r="L7" s="9" t="n">
+        <v>7561907.44</v>
+      </c>
+      <c r="M7" s="9" t="n">
+        <v>292548.17</v>
+      </c>
+      <c r="N7" s="9" t="n">
+        <v>822533.66</v>
+      </c>
+      <c r="O7" s="9" t="n">
+        <v>9005629.640000001</v>
+      </c>
+      <c r="P7" s="9" t="n">
+        <v>13080537.68</v>
+      </c>
+      <c r="Q7" s="9" t="n">
+        <v>440136137.2</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>2026-08-06</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="n">
+        <v>1180000000</v>
+      </c>
+      <c r="C8" s="6" t="n">
+        <v>142486082.56</v>
+      </c>
+      <c r="D8" s="6" t="n">
+        <v>18363859.9</v>
+      </c>
+      <c r="E8" s="6" t="n">
+        <v>655143</v>
+      </c>
+      <c r="F8" s="6" t="n">
+        <v>5010366.56</v>
+      </c>
+      <c r="G8" s="6" t="n">
+        <v>34132045</v>
+      </c>
+      <c r="H8" s="6" t="n">
+        <v>23846968</v>
+      </c>
+      <c r="I8" s="7" t="n">
+        <v>1404494465.02</v>
+      </c>
+      <c r="J8" s="8" t="n">
+        <v>327568000</v>
+      </c>
+      <c r="K8" s="9" t="n">
+        <v>50721504.22</v>
+      </c>
+      <c r="L8" s="9" t="n">
+        <v>7229157.84</v>
+      </c>
+      <c r="M8" s="9" t="n">
+        <v>314539.43</v>
+      </c>
+      <c r="N8" s="9" t="n">
+        <v>1460046.62</v>
+      </c>
+      <c r="O8" s="9" t="n">
+        <v>9946253.73</v>
+      </c>
+      <c r="P8" s="9" t="n">
+        <v>12037420</v>
+      </c>
+      <c r="Q8" s="9" t="n">
+        <v>409276921.85</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>2026-08-07</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="n">
+        <v>1160000000</v>
+      </c>
+      <c r="C9" s="6" t="n">
+        <v>119155726.68</v>
+      </c>
+      <c r="D9" s="6" t="n">
+        <v>15826632.35</v>
+      </c>
+      <c r="E9" s="6" t="n">
+        <v>614652</v>
+      </c>
+      <c r="F9" s="6" t="n">
+        <v>3319144.65</v>
+      </c>
+      <c r="G9" s="6" t="n">
+        <v>28308461</v>
+      </c>
+      <c r="H9" s="6" t="n">
+        <v>18491780</v>
+      </c>
+      <c r="I9" s="7" t="n">
+        <v>1345716396.68</v>
+      </c>
+      <c r="J9" s="8" t="n">
+        <v>322016000</v>
+      </c>
+      <c r="K9" s="9" t="n">
+        <v>45150709.09</v>
+      </c>
+      <c r="L9" s="9" t="n">
+        <v>4663406.57</v>
+      </c>
+      <c r="M9" s="9" t="n">
+        <v>280061.26</v>
+      </c>
+      <c r="N9" s="9" t="n">
+        <v>962433.0699999999</v>
+      </c>
+      <c r="O9" s="9" t="n">
+        <v>8208439.79</v>
+      </c>
+      <c r="P9" s="9" t="n">
+        <v>8928506.67</v>
+      </c>
+      <c r="Q9" s="9" t="n">
+        <v>390209556.44</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>2026-08-08</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="n">
+        <v>1290000000</v>
+      </c>
+      <c r="C10" s="6" t="n">
+        <v>119826023.15</v>
+      </c>
+      <c r="D10" s="6" t="n">
+        <v>20822561.28</v>
+      </c>
+      <c r="E10" s="6" t="n">
+        <v>1178183</v>
+      </c>
+      <c r="F10" s="6" t="n">
+        <v>9583995.710000001</v>
+      </c>
+      <c r="G10" s="6" t="n">
+        <v>31048172</v>
+      </c>
+      <c r="H10" s="6" t="n">
+        <v>23442223</v>
+      </c>
+      <c r="I10" s="7" t="n">
+        <v>1495901158.14</v>
+      </c>
+      <c r="J10" s="8" t="n">
+        <v>358104000</v>
+      </c>
+      <c r="K10" s="9" t="n">
+        <v>44119482.44</v>
+      </c>
+      <c r="L10" s="9" t="n">
+        <v>7466670.66</v>
+      </c>
+      <c r="M10" s="9" t="n">
+        <v>545929.65</v>
+      </c>
+      <c r="N10" s="9" t="n">
+        <v>2778971.06</v>
+      </c>
+      <c r="O10" s="9" t="n">
+        <v>9002713.9</v>
+      </c>
+      <c r="P10" s="9" t="n">
+        <v>11733055.02</v>
+      </c>
+      <c r="Q10" s="9" t="n">
+        <v>433750822.73</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>2026-08-09</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="n">
+        <v>1170000000</v>
+      </c>
+      <c r="C11" s="6" t="n">
+        <v>126747740.75</v>
+      </c>
+      <c r="D11" s="6" t="n">
+        <v>18043033.81</v>
+      </c>
+      <c r="E11" s="6" t="n">
+        <v>936332</v>
+      </c>
+      <c r="F11" s="6" t="n">
+        <v>9966584.189999999</v>
+      </c>
+      <c r="G11" s="6" t="n">
+        <v>36116656</v>
+      </c>
+      <c r="H11" s="6" t="n">
+        <v>34090206</v>
+      </c>
+      <c r="I11" s="7" t="n">
+        <v>1395900552.75</v>
+      </c>
+      <c r="J11" s="8" t="n">
+        <v>324792000</v>
+      </c>
+      <c r="K11" s="9" t="n">
+        <v>48633763.9</v>
+      </c>
+      <c r="L11" s="9" t="n">
+        <v>6159576.07</v>
+      </c>
+      <c r="M11" s="9" t="n">
+        <v>391311.2</v>
+      </c>
+      <c r="N11" s="9" t="n">
+        <v>2932449.05</v>
+      </c>
+      <c r="O11" s="9" t="n">
+        <v>10626534.78</v>
+      </c>
+      <c r="P11" s="9" t="n">
+        <v>17177521.22</v>
+      </c>
+      <c r="Q11" s="9" t="n">
+        <v>410713156.22</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="n">
+        <v>861600000</v>
+      </c>
+      <c r="C12" s="6" t="n">
+        <v>77414257.48</v>
+      </c>
+      <c r="D12" s="6" t="n">
+        <v>16189968.12</v>
+      </c>
+      <c r="E12" s="6" t="n">
+        <v>315621</v>
+      </c>
+      <c r="F12" s="6" t="n">
+        <v>7862717.9</v>
+      </c>
+      <c r="G12" s="6" t="n">
+        <v>14896086</v>
+      </c>
+      <c r="H12" s="6" t="n">
+        <v>11570724</v>
+      </c>
+      <c r="I12" s="7" t="n">
+        <v>989849374.5</v>
+      </c>
+      <c r="J12" s="8" t="n">
+        <v>239180160</v>
+      </c>
+      <c r="K12" s="9" t="n">
+        <v>28257376.93</v>
+      </c>
+      <c r="L12" s="9" t="n">
+        <v>5783341.08</v>
+      </c>
+      <c r="M12" s="9" t="n">
+        <v>146839.93</v>
+      </c>
+      <c r="N12" s="9" t="n">
+        <v>2270517.48</v>
+      </c>
+      <c r="O12" s="9" t="n">
+        <v>4301543.57</v>
+      </c>
+      <c r="P12" s="9" t="n">
+        <v>5899079.07</v>
+      </c>
+      <c r="Q12" s="9" t="n">
+        <v>285838858.06</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="n">
+        <v>1180000000</v>
+      </c>
+      <c r="C13" s="6" t="n">
+        <v>88962184</v>
+      </c>
+      <c r="D13" s="6" t="n">
+        <v>20926301.85</v>
+      </c>
+      <c r="E13" s="6" t="n">
+        <v>737122</v>
+      </c>
+      <c r="F13" s="6" t="n">
+        <v>10423439.05</v>
+      </c>
+      <c r="G13" s="6" t="n">
+        <v>22104454</v>
+      </c>
+      <c r="H13" s="6" t="n">
+        <v>20000913</v>
+      </c>
+      <c r="I13" s="7" t="n">
+        <v>1343154413.9</v>
+      </c>
+      <c r="J13" s="8" t="n">
+        <v>327568000</v>
+      </c>
+      <c r="K13" s="9" t="n">
+        <v>32891944.15</v>
+      </c>
+      <c r="L13" s="9" t="n">
+        <v>8237000.57</v>
+      </c>
+      <c r="M13" s="9" t="n">
+        <v>342568.77</v>
+      </c>
+      <c r="N13" s="9" t="n">
+        <v>3012908.88</v>
+      </c>
+      <c r="O13" s="9" t="n">
+        <v>6389321.75</v>
+      </c>
+      <c r="P13" s="9" t="n">
+        <v>9798821.01</v>
+      </c>
+      <c r="Q13" s="9" t="n">
+        <v>388240565.14</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="n">
+        <v>1300000000</v>
+      </c>
+      <c r="C14" s="6" t="n">
+        <v>115992580.3</v>
+      </c>
+      <c r="D14" s="6" t="n">
+        <v>22182572.72</v>
+      </c>
+      <c r="E14" s="6" t="n">
+        <v>957673</v>
+      </c>
+      <c r="F14" s="6" t="n">
+        <v>11663866.53</v>
+      </c>
+      <c r="G14" s="6" t="n">
+        <v>28925281</v>
+      </c>
+      <c r="H14" s="6" t="n">
+        <v>24439775</v>
+      </c>
+      <c r="I14" s="7" t="n">
+        <v>1504161748.55</v>
+      </c>
+      <c r="J14" s="8" t="n">
+        <v>360880000</v>
+      </c>
+      <c r="K14" s="9" t="n">
+        <v>44498190.03</v>
+      </c>
+      <c r="L14" s="9" t="n">
+        <v>8739413.83</v>
+      </c>
+      <c r="M14" s="9" t="n">
+        <v>463531.04</v>
+      </c>
+      <c r="N14" s="9" t="n">
+        <v>3398429.19</v>
+      </c>
+      <c r="O14" s="9" t="n">
+        <v>8427781.550000001</v>
+      </c>
+      <c r="P14" s="9" t="n">
+        <v>11851028.97</v>
+      </c>
+      <c r="Q14" s="9" t="n">
+        <v>438258374.61</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="n">
+        <v>1220000000</v>
+      </c>
+      <c r="C15" s="6" t="n">
+        <v>131352520.44</v>
+      </c>
+      <c r="D15" s="6" t="n">
+        <v>19980748.26</v>
+      </c>
+      <c r="E15" s="6" t="n">
+        <v>839703</v>
+      </c>
+      <c r="F15" s="6" t="n">
+        <v>15012128.02</v>
+      </c>
+      <c r="G15" s="6" t="n">
+        <v>31735376</v>
+      </c>
+      <c r="H15" s="6" t="n">
+        <v>24750783</v>
+      </c>
+      <c r="I15" s="7" t="n">
+        <v>1443671258.72</v>
+      </c>
+      <c r="J15" s="8" t="n">
+        <v>338672000</v>
+      </c>
+      <c r="K15" s="9" t="n">
+        <v>47657304.2</v>
+      </c>
+      <c r="L15" s="9" t="n">
+        <v>6578982.54</v>
+      </c>
+      <c r="M15" s="9" t="n">
+        <v>401500.01</v>
+      </c>
+      <c r="N15" s="9" t="n">
+        <v>4351229.76</v>
+      </c>
+      <c r="O15" s="9" t="n">
+        <v>9198423.59</v>
+      </c>
+      <c r="P15" s="9" t="n">
+        <v>11585255.98</v>
+      </c>
+      <c r="Q15" s="9" t="n">
+        <v>418444696.08</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="n">
+        <v>1200000000</v>
+      </c>
+      <c r="C16" s="6" t="n">
+        <v>123254387.3</v>
+      </c>
+      <c r="D16" s="6" t="n">
+        <v>21714770.99</v>
+      </c>
+      <c r="E16" s="6" t="n">
+        <v>1294705</v>
+      </c>
+      <c r="F16" s="6" t="n">
+        <v>13855386.15</v>
+      </c>
+      <c r="G16" s="6" t="n">
+        <v>29755699</v>
+      </c>
+      <c r="H16" s="6" t="n">
+        <v>13982284</v>
+      </c>
+      <c r="I16" s="7" t="n">
+        <v>1403857232.44</v>
+      </c>
+      <c r="J16" s="8" t="n">
+        <v>333120000</v>
+      </c>
+      <c r="K16" s="9" t="n">
+        <v>45100146.59</v>
+      </c>
+      <c r="L16" s="9" t="n">
+        <v>6848767.95</v>
+      </c>
+      <c r="M16" s="9" t="n">
+        <v>598777.14</v>
+      </c>
+      <c r="N16" s="9" t="n">
+        <v>3990201.72</v>
+      </c>
+      <c r="O16" s="9" t="n">
+        <v>8569320.26</v>
+      </c>
+      <c r="P16" s="9" t="n">
+        <v>6068522.46</v>
+      </c>
+      <c r="Q16" s="9" t="n">
+        <v>404295736.12</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="n">
+        <v>1500000000</v>
+      </c>
+      <c r="C17" s="6" t="n">
+        <v>135734087.98</v>
+      </c>
+      <c r="D17" s="6" t="n">
+        <v>26328429.67</v>
+      </c>
+      <c r="E17" s="6" t="n">
+        <v>2039246</v>
+      </c>
+      <c r="F17" s="6" t="n">
+        <v>17116844.44</v>
+      </c>
+      <c r="G17" s="6" t="n">
+        <v>38789476</v>
+      </c>
+      <c r="H17" s="6" t="n">
+        <v>23809525</v>
+      </c>
+      <c r="I17" s="7" t="n">
+        <v>1743817609.09</v>
+      </c>
+      <c r="J17" s="8" t="n">
+        <v>416400000</v>
+      </c>
+      <c r="K17" s="9" t="n">
+        <v>49047089.99</v>
+      </c>
+      <c r="L17" s="9" t="n">
+        <v>8232801.42</v>
+      </c>
+      <c r="M17" s="9" t="n">
+        <v>899431.51</v>
+      </c>
+      <c r="N17" s="9" t="n">
+        <v>4926149.54</v>
+      </c>
+      <c r="O17" s="9" t="n">
+        <v>11163433.78</v>
+      </c>
+      <c r="P17" s="9" t="n">
+        <v>11193826.09</v>
+      </c>
+      <c r="Q17" s="9" t="n">
+        <v>501862732.34</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t>2026-08-16</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="n">
+        <v>1400000000</v>
+      </c>
+      <c r="C18" s="6" t="n">
+        <v>147219414.75</v>
+      </c>
+      <c r="D18" s="6" t="n">
+        <v>20291070.01</v>
+      </c>
+      <c r="E18" s="6" t="n">
+        <v>1359591</v>
+      </c>
+      <c r="F18" s="6" t="n">
+        <v>14195115.2</v>
+      </c>
+      <c r="G18" s="6" t="n">
+        <v>45793344</v>
+      </c>
+      <c r="H18" s="6" t="n">
+        <v>24504254</v>
+      </c>
+      <c r="I18" s="7" t="n">
+        <v>1653362788.96</v>
+      </c>
+      <c r="J18" s="8" t="n">
+        <v>388640000</v>
+      </c>
+      <c r="K18" s="9" t="n">
+        <v>57064827.84</v>
+      </c>
+      <c r="L18" s="9" t="n">
+        <v>5253664.07</v>
+      </c>
+      <c r="M18" s="9" t="n">
+        <v>644960.33</v>
+      </c>
+      <c r="N18" s="9" t="n">
+        <v>4126757.68</v>
+      </c>
+      <c r="O18" s="9" t="n">
+        <v>13312891.88</v>
+      </c>
+      <c r="P18" s="9" t="n">
+        <v>11617145.57</v>
+      </c>
+      <c r="Q18" s="9" t="n">
+        <v>480660247.37</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t>2026-08-17</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="n">
+        <v>926400000</v>
+      </c>
+      <c r="C19" s="6" t="n">
+        <v>101346609.5</v>
+      </c>
+      <c r="D19" s="6" t="n">
+        <v>17248459.41</v>
+      </c>
+      <c r="E19" s="6" t="n">
+        <v>1210622</v>
+      </c>
+      <c r="F19" s="6" t="n">
+        <v>11337468.16</v>
+      </c>
+      <c r="G19" s="6" t="n">
+        <v>19897635</v>
+      </c>
+      <c r="H19" s="6" t="n">
+        <v>11943453</v>
+      </c>
+      <c r="I19" s="7" t="n">
+        <v>1089384247.07</v>
+      </c>
+      <c r="J19" s="8" t="n">
+        <v>257168640</v>
+      </c>
+      <c r="K19" s="9" t="n">
+        <v>37038769.64</v>
+      </c>
+      <c r="L19" s="9" t="n">
+        <v>6582665.07</v>
+      </c>
+      <c r="M19" s="9" t="n">
+        <v>587784.12</v>
+      </c>
+      <c r="N19" s="9" t="n">
+        <v>3288970.22</v>
+      </c>
+      <c r="O19" s="9" t="n">
+        <v>5772252.5</v>
+      </c>
+      <c r="P19" s="9" t="n">
+        <v>5588473.52</v>
+      </c>
+      <c r="Q19" s="9" t="n">
+        <v>316027555.06</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="4" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="B20" s="5" t="n">
+        <v>1160000000</v>
+      </c>
+      <c r="C20" s="6" t="n">
+        <v>105672875.16</v>
+      </c>
+      <c r="D20" s="6" t="n">
+        <v>20729166.99</v>
+      </c>
+      <c r="E20" s="6" t="n">
+        <v>557181</v>
+      </c>
+      <c r="F20" s="6" t="n">
+        <v>12627740.01</v>
+      </c>
+      <c r="G20" s="6" t="n">
+        <v>25712157</v>
+      </c>
+      <c r="H20" s="6" t="n">
+        <v>14893199</v>
+      </c>
+      <c r="I20" s="7" t="n">
+        <v>1340192319.16</v>
+      </c>
+      <c r="J20" s="8" t="n">
+        <v>322016000</v>
+      </c>
+      <c r="K20" s="9" t="n">
+        <v>38155857.92</v>
+      </c>
+      <c r="L20" s="9" t="n">
+        <v>7373273.33</v>
+      </c>
+      <c r="M20" s="9" t="n">
+        <v>262338.04</v>
+      </c>
+      <c r="N20" s="9" t="n">
+        <v>3635012.06</v>
+      </c>
+      <c r="O20" s="9" t="n">
+        <v>7401482.81</v>
+      </c>
+      <c r="P20" s="9" t="n">
+        <v>6942822.13</v>
+      </c>
+      <c r="Q20" s="9" t="n">
+        <v>385786786.29</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="4" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="B21" s="5" t="n">
+        <v>1370000000</v>
+      </c>
+      <c r="C21" s="6" t="n">
+        <v>124084423.03</v>
+      </c>
+      <c r="D21" s="6" t="n">
+        <v>23043283.69</v>
+      </c>
+      <c r="E21" s="6" t="n">
+        <v>1450093</v>
+      </c>
+      <c r="F21" s="6" t="n">
+        <v>15105978.17</v>
+      </c>
+      <c r="G21" s="6" t="n">
+        <v>32106553</v>
+      </c>
+      <c r="H21" s="6" t="n">
+        <v>21675050</v>
+      </c>
+      <c r="I21" s="7" t="n">
+        <v>1587465380.89</v>
+      </c>
+      <c r="J21" s="8" t="n">
+        <v>380312000</v>
+      </c>
+      <c r="K21" s="9" t="n">
+        <v>44959266.73</v>
+      </c>
+      <c r="L21" s="9" t="n">
+        <v>7699311.71</v>
+      </c>
+      <c r="M21" s="9" t="n">
+        <v>691813.04</v>
+      </c>
+      <c r="N21" s="9" t="n">
+        <v>4356201.81</v>
+      </c>
+      <c r="O21" s="9" t="n">
+        <v>9258759.859999999</v>
+      </c>
+      <c r="P21" s="9" t="n">
+        <v>10509589.79</v>
+      </c>
+      <c r="Q21" s="9" t="n">
+        <v>457786942.94</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="4" t="inlineStr">
+        <is>
+          <t>2026-08-20</t>
+        </is>
+      </c>
+      <c r="B22" s="5" t="n">
+        <v>1190000000</v>
+      </c>
+      <c r="C22" s="6" t="n">
+        <v>133614522.35</v>
+      </c>
+      <c r="D22" s="6" t="n">
+        <v>19460265.91</v>
+      </c>
+      <c r="E22" s="6" t="n">
+        <v>895848</v>
+      </c>
+      <c r="F22" s="6" t="n">
+        <v>13770677.81</v>
+      </c>
+      <c r="G22" s="6" t="n">
+        <v>32240466</v>
+      </c>
+      <c r="H22" s="6" t="n">
+        <v>25089021</v>
+      </c>
+      <c r="I22" s="7" t="n">
+        <v>1415070801.07</v>
+      </c>
+      <c r="J22" s="8" t="n">
+        <v>330344000</v>
+      </c>
+      <c r="K22" s="9" t="n">
+        <v>44531856.81</v>
+      </c>
+      <c r="L22" s="9" t="n">
+        <v>5997303.28</v>
+      </c>
+      <c r="M22" s="9" t="n">
+        <v>426029.96</v>
+      </c>
+      <c r="N22" s="9" t="n">
+        <v>3953306.49</v>
+      </c>
+      <c r="O22" s="9" t="n">
+        <v>9255640.52</v>
+      </c>
+      <c r="P22" s="9" t="n">
+        <v>11732475.1</v>
+      </c>
+      <c r="Q22" s="9" t="n">
+        <v>406240612.16</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="4" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="B23" s="5" t="n">
+        <v>1260000000</v>
+      </c>
+      <c r="C23" s="6" t="n">
+        <v>119176847.25</v>
+      </c>
+      <c r="D23" s="6" t="n">
+        <v>22591885.42</v>
+      </c>
+      <c r="E23" s="6" t="n">
+        <v>1198992</v>
+      </c>
+      <c r="F23" s="6" t="n">
+        <v>16590934.97</v>
+      </c>
+      <c r="G23" s="6" t="n">
+        <v>28572335</v>
+      </c>
+      <c r="H23" s="6" t="n">
+        <v>9902841</v>
+      </c>
+      <c r="I23" s="7" t="n">
+        <v>1458033835.64</v>
+      </c>
+      <c r="J23" s="8" t="n">
+        <v>349776000</v>
+      </c>
+      <c r="K23" s="9" t="n">
+        <v>35238750.52</v>
+      </c>
+      <c r="L23" s="9" t="n">
+        <v>9390952.41</v>
+      </c>
+      <c r="M23" s="9" t="n">
+        <v>577229.27</v>
+      </c>
+      <c r="N23" s="9" t="n">
+        <v>4682007.62</v>
+      </c>
+      <c r="O23" s="9" t="n">
+        <v>8063191.77</v>
+      </c>
+      <c r="P23" s="9" t="n">
+        <v>3733039.67</v>
+      </c>
+      <c r="Q23" s="9" t="n">
+        <v>411461171.27</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="4" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
+        </is>
+      </c>
+      <c r="B24" s="5" t="n">
+        <v>1680000000</v>
+      </c>
+      <c r="C24" s="6" t="n">
+        <v>147197041.73</v>
+      </c>
+      <c r="D24" s="6" t="n">
+        <v>34454101.03</v>
+      </c>
+      <c r="E24" s="6" t="n">
+        <v>1122513</v>
+      </c>
+      <c r="F24" s="6" t="n">
+        <v>25849266.6</v>
+      </c>
+      <c r="G24" s="6" t="n">
+        <v>44528557</v>
+      </c>
+      <c r="H24" s="6" t="n">
+        <v>21274756</v>
+      </c>
+      <c r="I24" s="7" t="n">
+        <v>1954426235.36</v>
+      </c>
+      <c r="J24" s="8" t="n">
+        <v>466368000</v>
+      </c>
+      <c r="K24" s="9" t="n">
+        <v>43368591.4</v>
+      </c>
+      <c r="L24" s="9" t="n">
+        <v>11415691.98</v>
+      </c>
+      <c r="M24" s="9" t="n">
+        <v>545961.96</v>
+      </c>
+      <c r="N24" s="9" t="n">
+        <v>7290541.98</v>
+      </c>
+      <c r="O24" s="9" t="n">
+        <v>12558859.76</v>
+      </c>
+      <c r="P24" s="9" t="n">
+        <v>9679849.300000001</v>
+      </c>
+      <c r="Q24" s="9" t="n">
+        <v>551227496.37</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="4" t="inlineStr">
+        <is>
+          <t>2026-08-23</t>
+        </is>
+      </c>
+      <c r="B25" s="5" t="n">
+        <v>1480000000</v>
+      </c>
+      <c r="C25" s="6" t="n">
+        <v>145329668.29</v>
+      </c>
+      <c r="D25" s="6" t="n">
+        <v>25659770.52</v>
+      </c>
+      <c r="E25" s="6" t="n">
+        <v>1532660</v>
+      </c>
+      <c r="F25" s="6" t="n">
+        <v>16408150.57</v>
+      </c>
+      <c r="G25" s="6" t="n">
+        <v>44263912</v>
+      </c>
+      <c r="H25" s="6" t="n">
+        <v>21410910</v>
+      </c>
+      <c r="I25" s="7" t="n">
+        <v>1734605071.38</v>
+      </c>
+      <c r="J25" s="8" t="n">
+        <v>410848000</v>
+      </c>
+      <c r="K25" s="9" t="n">
+        <v>45347988.13</v>
+      </c>
+      <c r="L25" s="9" t="n">
+        <v>8441476.460000001</v>
+      </c>
+      <c r="M25" s="9" t="n">
+        <v>678289.72</v>
+      </c>
+      <c r="N25" s="9" t="n">
+        <v>4660735.14</v>
+      </c>
+      <c r="O25" s="9" t="n">
+        <v>12573164.11</v>
+      </c>
+      <c r="P25" s="9" t="n">
+        <v>10164913.41</v>
+      </c>
+      <c r="Q25" s="9" t="n">
+        <v>492714566.97</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="4" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+      <c r="B26" s="5" t="n">
+        <v>1120000000</v>
+      </c>
+      <c r="C26" s="6" t="n">
+        <v>98117953.89</v>
+      </c>
+      <c r="D26" s="6" t="n">
+        <v>21651553.57</v>
+      </c>
+      <c r="E26" s="6" t="n">
+        <v>525316</v>
+      </c>
+      <c r="F26" s="6" t="n">
+        <v>13798244.33</v>
+      </c>
+      <c r="G26" s="6" t="n">
+        <v>25729394</v>
+      </c>
+      <c r="H26" s="6" t="n">
+        <v>12004100</v>
+      </c>
+      <c r="I26" s="7" t="n">
+        <v>1291826561.79</v>
+      </c>
+      <c r="J26" s="8" t="n">
+        <v>310912000</v>
+      </c>
+      <c r="K26" s="9" t="n">
+        <v>31546614.61</v>
+      </c>
+      <c r="L26" s="9" t="n">
+        <v>6064427.21</v>
+      </c>
+      <c r="M26" s="9" t="n">
+        <v>240533.84</v>
+      </c>
+      <c r="N26" s="9" t="n">
+        <v>3901201.2</v>
+      </c>
+      <c r="O26" s="9" t="n">
+        <v>7274515.54</v>
+      </c>
+      <c r="P26" s="9" t="n">
+        <v>5301039.25</v>
+      </c>
+      <c r="Q26" s="9" t="n">
+        <v>365240331.65</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="4" t="inlineStr">
+        <is>
+          <t>2026-08-25</t>
+        </is>
+      </c>
+      <c r="B27" s="5" t="n">
+        <v>1320000000</v>
+      </c>
+      <c r="C27" s="6" t="n">
+        <v>122647932.15</v>
+      </c>
+      <c r="D27" s="6" t="n">
+        <v>25712632.31</v>
+      </c>
+      <c r="E27" s="6" t="n">
+        <v>689662</v>
+      </c>
+      <c r="F27" s="6" t="n">
+        <v>12631632.8</v>
+      </c>
+      <c r="G27" s="6" t="n">
+        <v>31326910</v>
+      </c>
+      <c r="H27" s="6" t="n">
+        <v>16941298</v>
+      </c>
+      <c r="I27" s="7" t="n">
+        <v>1529950067.26</v>
+      </c>
+      <c r="J27" s="8" t="n">
+        <v>366432000</v>
+      </c>
+      <c r="K27" s="9" t="n">
+        <v>38758367.74</v>
+      </c>
+      <c r="L27" s="9" t="n">
+        <v>7634695.65</v>
+      </c>
+      <c r="M27" s="9" t="n">
+        <v>345067.73</v>
+      </c>
+      <c r="N27" s="9" t="n">
+        <v>3577476.75</v>
+      </c>
+      <c r="O27" s="9" t="n">
+        <v>8872272.810000001</v>
+      </c>
+      <c r="P27" s="9" t="n">
+        <v>7686001.99</v>
+      </c>
+      <c r="Q27" s="9" t="n">
+        <v>433305882.68</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="4" t="inlineStr">
+        <is>
+          <t>2026-08-26</t>
+        </is>
+      </c>
+      <c r="B28" s="5" t="n">
+        <v>1420000000</v>
+      </c>
+      <c r="C28" s="6" t="n">
+        <v>146914840.72</v>
+      </c>
+      <c r="D28" s="6" t="n">
+        <v>26242191.02</v>
+      </c>
+      <c r="E28" s="6" t="n">
+        <v>2557592</v>
+      </c>
+      <c r="F28" s="6" t="n">
+        <v>11278878.58</v>
+      </c>
+      <c r="G28" s="6" t="n">
+        <v>38474611</v>
+      </c>
+      <c r="H28" s="6" t="n">
+        <v>23226558</v>
+      </c>
+      <c r="I28" s="7" t="n">
+        <v>1668694671.32</v>
+      </c>
+      <c r="J28" s="8" t="n">
+        <v>394192000</v>
+      </c>
+      <c r="K28" s="9" t="n">
+        <v>47966998.93</v>
+      </c>
+      <c r="L28" s="9" t="n">
+        <v>9260973.609999999</v>
+      </c>
+      <c r="M28" s="9" t="n">
+        <v>1170559.87</v>
+      </c>
+      <c r="N28" s="9" t="n">
+        <v>3227798.28</v>
+      </c>
+      <c r="O28" s="9" t="n">
+        <v>11010694.22</v>
+      </c>
+      <c r="P28" s="9" t="n">
+        <v>10719319.3</v>
+      </c>
+      <c r="Q28" s="9" t="n">
+        <v>477548344.21</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="4" t="inlineStr">
+        <is>
+          <t>2026-08-27</t>
+        </is>
+      </c>
+      <c r="B29" s="5" t="n">
+        <v>1190000000</v>
+      </c>
+      <c r="C29" s="6" t="n">
+        <v>111275220.48</v>
+      </c>
+      <c r="D29" s="6" t="n">
+        <v>18973251.97</v>
+      </c>
+      <c r="E29" s="6" t="n">
+        <v>9547705</v>
+      </c>
+      <c r="F29" s="6" t="n">
+        <v>12827436.18</v>
+      </c>
+      <c r="G29" s="6" t="n">
+        <v>30358401</v>
+      </c>
+      <c r="H29" s="6" t="n">
+        <v>23537141</v>
+      </c>
+      <c r="I29" s="7" t="n">
+        <v>1396519155.63</v>
+      </c>
+      <c r="J29" s="8" t="n">
+        <v>330344000</v>
+      </c>
+      <c r="K29" s="9" t="n">
+        <v>33561811.06</v>
+      </c>
+      <c r="L29" s="9" t="n">
+        <v>6610438.95</v>
+      </c>
+      <c r="M29" s="9" t="n">
+        <v>3504492.28</v>
+      </c>
+      <c r="N29" s="9" t="n">
+        <v>3640235.79</v>
+      </c>
+      <c r="O29" s="9" t="n">
+        <v>8615263.130000001</v>
+      </c>
+      <c r="P29" s="9" t="n">
+        <v>10035145.32</v>
+      </c>
+      <c r="Q29" s="9" t="n">
+        <v>396311386.54</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="4" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
+      </c>
+      <c r="B30" s="5" t="n">
+        <v>1490000000</v>
+      </c>
+      <c r="C30" s="6" t="n">
+        <v>98118727.63</v>
+      </c>
+      <c r="D30" s="6" t="n">
+        <v>28162072.11</v>
+      </c>
+      <c r="E30" s="6" t="n">
+        <v>14809135</v>
+      </c>
+      <c r="F30" s="6" t="n">
+        <v>18367442.31</v>
+      </c>
+      <c r="G30" s="6" t="n">
+        <v>21799182</v>
+      </c>
+      <c r="H30" s="6" t="n">
+        <v>15601449</v>
+      </c>
+      <c r="I30" s="7" t="n">
+        <v>1686858008.05</v>
+      </c>
+      <c r="J30" s="8" t="n">
+        <v>413624000</v>
+      </c>
+      <c r="K30" s="9" t="n">
+        <v>30240724.05</v>
+      </c>
+      <c r="L30" s="9" t="n">
+        <v>9490626.810000001</v>
+      </c>
+      <c r="M30" s="9" t="n">
+        <v>5547393.25</v>
+      </c>
+      <c r="N30" s="9" t="n">
+        <v>5188369.11</v>
+      </c>
+      <c r="O30" s="9" t="n">
+        <v>6157754.61</v>
+      </c>
+      <c r="P30" s="9" t="n">
+        <v>6248721.69</v>
+      </c>
+      <c r="Q30" s="9" t="n">
+        <v>476497589.52</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="4" t="inlineStr">
+        <is>
+          <t>2026-08-29</t>
+        </is>
+      </c>
+      <c r="B31" s="5" t="n">
+        <v>1930000000</v>
+      </c>
+      <c r="C31" s="6" t="n">
+        <v>165005629.65</v>
+      </c>
+      <c r="D31" s="6" t="n">
+        <v>34918943.24</v>
+      </c>
+      <c r="E31" s="6" t="n">
+        <v>28273980</v>
+      </c>
+      <c r="F31" s="6" t="n">
+        <v>18842311.25</v>
+      </c>
+      <c r="G31" s="6" t="n">
+        <v>29109748</v>
+      </c>
+      <c r="H31" s="6" t="n">
+        <v>26623498</v>
+      </c>
+      <c r="I31" s="7" t="n">
+        <v>2232774110.14</v>
+      </c>
+      <c r="J31" s="8" t="n">
+        <v>535768000</v>
+      </c>
+      <c r="K31" s="9" t="n">
+        <v>46829617.02</v>
+      </c>
+      <c r="L31" s="9" t="n">
+        <v>11632838.68</v>
+      </c>
+      <c r="M31" s="9" t="n">
+        <v>10477277.08</v>
+      </c>
+      <c r="N31" s="9" t="n">
+        <v>5320843.96</v>
+      </c>
+      <c r="O31" s="9" t="n">
+        <v>8220245.64</v>
+      </c>
+      <c r="P31" s="9" t="n">
+        <v>12259956.04</v>
+      </c>
+      <c r="Q31" s="9" t="n">
+        <v>630508778.4299999</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="4" t="inlineStr">
+        <is>
+          <t>2026-08-30</t>
+        </is>
+      </c>
+      <c r="B32" s="5" t="n">
+        <v>1700000000</v>
+      </c>
+      <c r="C32" s="6" t="n">
+        <v>153283200.98</v>
+      </c>
+      <c r="D32" s="6" t="n">
+        <v>25897044.82</v>
+      </c>
+      <c r="E32" s="6" t="n">
+        <v>4910082</v>
+      </c>
+      <c r="F32" s="6" t="n">
+        <v>13252847.35</v>
+      </c>
+      <c r="G32" s="6" t="n">
+        <v>33872270</v>
+      </c>
+      <c r="H32" s="6" t="n">
+        <v>31086830</v>
+      </c>
+      <c r="I32" s="7" t="n">
+        <v>1962302275.15</v>
+      </c>
+      <c r="J32" s="8" t="n">
+        <v>471920000</v>
+      </c>
+      <c r="K32" s="9" t="n">
+        <v>46033156.99</v>
+      </c>
+      <c r="L32" s="9" t="n">
+        <v>7924109.45</v>
+      </c>
+      <c r="M32" s="9" t="n">
+        <v>1721674.99</v>
+      </c>
+      <c r="N32" s="9" t="n">
+        <v>3750171.98</v>
+      </c>
+      <c r="O32" s="9" t="n">
+        <v>9584871.42</v>
+      </c>
+      <c r="P32" s="9" t="n">
+        <v>14340728.19</v>
+      </c>
+      <c r="Q32" s="9" t="n">
+        <v>555274713.02</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="4" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="B33" s="5" t="n">
+        <v>1400000000</v>
+      </c>
+      <c r="C33" s="6" t="n">
+        <v>113668391.39</v>
+      </c>
+      <c r="D33" s="6" t="n">
+        <v>24833122.69</v>
+      </c>
+      <c r="E33" s="6" t="n">
+        <v>15463</v>
+      </c>
+      <c r="F33" s="6" t="n">
+        <v>7051751.21</v>
+      </c>
+      <c r="G33" s="6" t="n">
+        <v>32256260</v>
+      </c>
+      <c r="H33" s="6" t="n">
+        <v>11845545</v>
+      </c>
+      <c r="I33" s="7" t="n">
+        <v>1589670533.29</v>
+      </c>
+      <c r="J33" s="8" t="n">
+        <v>388640000</v>
+      </c>
+      <c r="K33" s="9" t="n">
+        <v>36835334.14</v>
+      </c>
+      <c r="L33" s="9" t="n">
+        <v>8164954.36</v>
+      </c>
+      <c r="M33" s="9" t="n">
+        <v>7580.34</v>
+      </c>
+      <c r="N33" s="9" t="n">
+        <v>1997237.73</v>
+      </c>
+      <c r="O33" s="9" t="n">
+        <v>9135804.35</v>
+      </c>
+      <c r="P33" s="9" t="n">
+        <v>5454763.56</v>
+      </c>
+      <c r="Q33" s="9" t="n">
+        <v>450235674.48</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="B34" s="5" t="n">
+        <v>1520000000</v>
+      </c>
+      <c r="C34" s="6" t="n">
+        <v>111712158.6</v>
+      </c>
+      <c r="D34" s="6" t="n">
+        <v>30033982.35</v>
+      </c>
+      <c r="E34" s="6" t="n">
+        <v>17941206</v>
+      </c>
+      <c r="F34" s="6" t="n">
+        <v>5769286.27</v>
+      </c>
+      <c r="G34" s="6" t="n">
+        <v>42760798</v>
+      </c>
+      <c r="H34" s="6" t="n">
+        <v>19024989</v>
+      </c>
+      <c r="I34" s="7" t="n">
+        <v>1747242420.22</v>
+      </c>
+      <c r="J34" s="8" t="n">
+        <v>421952000</v>
+      </c>
+      <c r="K34" s="9" t="n">
+        <v>33675810.27</v>
+      </c>
+      <c r="L34" s="9" t="n">
+        <v>8422284.43</v>
+      </c>
+      <c r="M34" s="9" t="n">
+        <v>7000711.88</v>
+      </c>
+      <c r="N34" s="9" t="n">
+        <v>1629230.19</v>
+      </c>
+      <c r="O34" s="9" t="n">
+        <v>12075528.88</v>
+      </c>
+      <c r="P34" s="9" t="n">
+        <v>8660771.18</v>
+      </c>
+      <c r="Q34" s="9" t="n">
+        <v>493416336.83</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="B35" s="5" t="n">
+        <v>1580000000</v>
+      </c>
+      <c r="C35" s="6" t="n">
+        <v>133200326.87</v>
+      </c>
+      <c r="D35" s="6" t="n">
+        <v>26868942.32</v>
+      </c>
+      <c r="E35" s="6" t="n">
+        <v>21144810</v>
+      </c>
+      <c r="F35" s="6" t="n">
+        <v>9396009.67</v>
+      </c>
+      <c r="G35" s="6" t="n">
+        <v>30959003</v>
+      </c>
+      <c r="H35" s="6" t="n">
+        <v>25133206</v>
+      </c>
+      <c r="I35" s="7" t="n">
+        <v>1826702297.86</v>
+      </c>
+      <c r="J35" s="8" t="n">
+        <v>438608000</v>
+      </c>
+      <c r="K35" s="9" t="n">
+        <v>39150985.29</v>
+      </c>
+      <c r="L35" s="9" t="n">
+        <v>6948205.54</v>
+      </c>
+      <c r="M35" s="9" t="n">
+        <v>7686788.4</v>
+      </c>
+      <c r="N35" s="9" t="n">
+        <v>2654002.85</v>
+      </c>
+      <c r="O35" s="9" t="n">
+        <v>8744699.619999999</v>
+      </c>
+      <c r="P35" s="9" t="n">
+        <v>12178807.65</v>
+      </c>
+      <c r="Q35" s="9" t="n">
+        <v>515971489.35</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+      <c r="B36" s="5" t="n">
+        <v>1540000000</v>
+      </c>
+      <c r="C36" s="6" t="n">
+        <v>148468892.52</v>
+      </c>
+      <c r="D36" s="6" t="n">
+        <v>27279175.53</v>
+      </c>
+      <c r="E36" s="6" t="n">
+        <v>24810710</v>
+      </c>
+      <c r="F36" s="6" t="n">
+        <v>10391420.59</v>
+      </c>
+      <c r="G36" s="6" t="n">
+        <v>31438450.5</v>
+      </c>
+      <c r="H36" s="6" t="n">
+        <v>28258944</v>
+      </c>
+      <c r="I36" s="7" t="n">
+        <v>1810647593.14</v>
+      </c>
+      <c r="J36" s="8" t="n">
+        <v>427504000</v>
+      </c>
+      <c r="K36" s="9" t="n">
+        <v>47297561.25</v>
+      </c>
+      <c r="L36" s="9" t="n">
+        <v>9261586.119999999</v>
+      </c>
+      <c r="M36" s="9" t="n">
+        <v>8799940.630000001</v>
+      </c>
+      <c r="N36" s="9" t="n">
+        <v>2976367.39</v>
+      </c>
+      <c r="O36" s="9" t="n">
+        <v>9004772.539999999</v>
+      </c>
+      <c r="P36" s="9" t="n">
+        <v>13771335.88</v>
+      </c>
+      <c r="Q36" s="9" t="n">
+        <v>518615563.81</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="B37" s="5" t="n">
+        <v>1523154175.75</v>
+      </c>
+      <c r="C37" s="6" t="n">
+        <v>162404936.11</v>
+      </c>
+      <c r="D37" s="6" t="n">
+        <v>32818984.23</v>
+      </c>
+      <c r="E37" s="6" t="n">
+        <v>20593115</v>
+      </c>
+      <c r="F37" s="6" t="n">
+        <v>10350317.52</v>
+      </c>
+      <c r="G37" s="6" t="n">
+        <v>38546740</v>
+      </c>
+      <c r="H37" s="6" t="n">
+        <v>14064111</v>
+      </c>
+      <c r="I37" s="7" t="n">
+        <v>1801932379.61</v>
+      </c>
+      <c r="J37" s="8" t="n">
+        <v>422827599.19</v>
+      </c>
+      <c r="K37" s="9" t="n">
+        <v>50100849.41</v>
+      </c>
+      <c r="L37" s="9" t="n">
+        <v>10372615.86</v>
+      </c>
+      <c r="M37" s="9" t="n">
+        <v>7004156.33</v>
+      </c>
+      <c r="N37" s="9" t="n">
+        <v>2931559.34</v>
+      </c>
+      <c r="O37" s="9" t="n">
+        <v>10917738.06</v>
+      </c>
+      <c r="P37" s="9" t="n">
+        <v>6213562.76</v>
+      </c>
+      <c r="Q37" s="9" t="n">
+        <v>510368080.94</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-05</t>
+        </is>
+      </c>
+      <c r="B38" s="5" t="n"/>
+      <c r="C38" s="6" t="n">
+        <v>173014888.85</v>
+      </c>
+      <c r="D38" s="6" t="n">
+        <v>50137129.16</v>
+      </c>
+      <c r="E38" s="6" t="n">
+        <v>52782942</v>
+      </c>
+      <c r="F38" s="6" t="n">
+        <v>17867253.73</v>
+      </c>
+      <c r="G38" s="6" t="n">
+        <v>31935868</v>
+      </c>
+      <c r="H38" s="6" t="n">
+        <v>21111711</v>
+      </c>
+      <c r="I38" s="7" t="n">
+        <v>346849792.74</v>
+      </c>
+      <c r="J38" s="8" t="n"/>
+      <c r="K38" s="9" t="n">
+        <v>46914612.74</v>
+      </c>
+      <c r="L38" s="9" t="n">
+        <v>18023125.75</v>
+      </c>
+      <c r="M38" s="9" t="n">
+        <v>15883449.41</v>
+      </c>
+      <c r="N38" s="9" t="n">
+        <v>5459538.21</v>
+      </c>
+      <c r="O38" s="9" t="n">
+        <v>9758359.859999999</v>
+      </c>
+      <c r="P38" s="9" t="n">
+        <v>9944728.02</v>
+      </c>
+      <c r="Q38" s="9" t="n">
+        <v>105983813.98</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="B39" s="5" t="n"/>
+      <c r="C39" s="6" t="n">
+        <v>132077170.89</v>
+      </c>
+      <c r="D39" s="6" t="n">
+        <v>32056055.97</v>
+      </c>
+      <c r="E39" s="6" t="n">
+        <v>35925674</v>
+      </c>
+      <c r="F39" s="6" t="n">
+        <v>21673332.38</v>
+      </c>
+      <c r="G39" s="6" t="n">
+        <v>34863515</v>
+      </c>
+      <c r="H39" s="6" t="n">
+        <v>33781884</v>
+      </c>
+      <c r="I39" s="7" t="n">
+        <v>290377632.24</v>
+      </c>
+      <c r="J39" s="8" t="n"/>
+      <c r="K39" s="9" t="n">
+        <v>38188228.54</v>
+      </c>
+      <c r="L39" s="9" t="n">
+        <v>13010644.31</v>
+      </c>
+      <c r="M39" s="9" t="n">
+        <v>11501420.69</v>
+      </c>
+      <c r="N39" s="9" t="n">
+        <v>7315628</v>
+      </c>
+      <c r="O39" s="9" t="n">
+        <v>11767849.17</v>
+      </c>
+      <c r="P39" s="9" t="n">
+        <v>16230447.81</v>
+      </c>
+      <c r="Q39" s="9" t="n">
+        <v>98014218.51000001</v>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A2:Q39"/>
+  <mergeCells count="2">
+    <mergeCell ref="B1:I1"/>
+    <mergeCell ref="J1:Q1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:M41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2728,7 +4932,7 @@
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
-          <t>Combo / parlay share of that venue</t>
+          <t>Combo / parlay share of that venue's sports book</t>
         </is>
       </c>
     </row>
@@ -2822,7 +5026,7 @@
         <v>15122319</v>
       </c>
       <c r="H3" s="11" t="n">
-        <v>0.4816</v>
+        <v>0.5537</v>
       </c>
       <c r="I3" s="11" t="n"/>
       <c r="J3" s="11" t="n">
@@ -2861,7 +5065,7 @@
         <v>13414300</v>
       </c>
       <c r="H4" s="11" t="n">
-        <v>0.4816</v>
+        <v>0.5855</v>
       </c>
       <c r="I4" s="11" t="n"/>
       <c r="J4" s="11" t="n">
@@ -2900,7 +5104,7 @@
         <v>5593903</v>
       </c>
       <c r="H5" s="11" t="n">
-        <v>0.4816</v>
+        <v>0.5191</v>
       </c>
       <c r="I5" s="11" t="n"/>
       <c r="J5" s="11" t="n">
@@ -2941,7 +5145,7 @@
         <v>10388004</v>
       </c>
       <c r="H6" s="11" t="n">
-        <v>0.4816</v>
+        <v>0.5629</v>
       </c>
       <c r="I6" s="11" t="n">
         <v>0.3931</v>
@@ -2984,7 +5188,7 @@
         <v>11554341</v>
       </c>
       <c r="H7" s="11" t="n">
-        <v>0.4816</v>
+        <v>0.5704</v>
       </c>
       <c r="I7" s="11" t="n">
         <v>0.3082</v>
@@ -3027,7 +5231,7 @@
         <v>11900005</v>
       </c>
       <c r="H8" s="11" t="n">
-        <v>0.4816</v>
+        <v>0.5618</v>
       </c>
       <c r="I8" s="11" t="n">
         <v>0.3006</v>
@@ -3070,7 +5274,7 @@
         <v>9881154</v>
       </c>
       <c r="H9" s="11" t="n">
-        <v>0.4816</v>
+        <v>0.5807</v>
       </c>
       <c r="I9" s="11" t="n">
         <v>0.3517</v>
@@ -3113,7 +5317,7 @@
         <v>12561820</v>
       </c>
       <c r="H10" s="11" t="n">
-        <v>0.4816</v>
+        <v>0.5789</v>
       </c>
       <c r="I10" s="11" t="n">
         <v>0.3298</v>
@@ -3156,7 +5360,7 @@
         <v>12447288</v>
       </c>
       <c r="H11" s="11" t="n">
-        <v>0.4816</v>
+        <v>0.5864</v>
       </c>
       <c r="I11" s="11" t="n">
         <v>0.3287</v>
@@ -3199,7 +5403,7 @@
         <v>5158036</v>
       </c>
       <c r="H12" s="11" t="n">
-        <v>0.4816</v>
+        <v>0.6043999999999999</v>
       </c>
       <c r="I12" s="11" t="n">
         <v>0.3621</v>
@@ -3242,7 +5446,7 @@
         <v>9937864</v>
       </c>
       <c r="H13" s="11" t="n">
-        <v>0.4816</v>
+        <v>0.5853</v>
       </c>
       <c r="I13" s="11" t="n">
         <v>0.3335</v>
@@ -3285,7 +5489,7 @@
         <v>11483868</v>
       </c>
       <c r="H14" s="11" t="n">
-        <v>0.4816</v>
+        <v>0.6004</v>
       </c>
       <c r="I14" s="11" t="n">
         <v>0.3297</v>
@@ -3328,7 +5532,7 @@
         <v>11876717</v>
       </c>
       <c r="H15" s="11" t="n">
-        <v>0.4816</v>
+        <v>0.5614</v>
       </c>
       <c r="I15" s="11" t="n">
         <v>0.3308</v>
@@ -3371,7 +5575,7 @@
         <v>10105691</v>
       </c>
       <c r="H16" s="11" t="n">
-        <v>0.4816</v>
+        <v>0.5629</v>
       </c>
       <c r="I16" s="11" t="n">
         <v>0.3907</v>
@@ -3414,7 +5618,7 @@
         <v>15529922</v>
       </c>
       <c r="H17" s="11" t="n">
-        <v>0.4816</v>
+        <v>0.5665</v>
       </c>
       <c r="I17" s="11" t="n">
         <v>0.3994</v>
@@ -3457,7 +5661,7 @@
         <v>16183161</v>
       </c>
       <c r="H18" s="11" t="n">
-        <v>0.4816</v>
+        <v>0.6003000000000001</v>
       </c>
       <c r="I18" s="11" t="n">
         <v>0.3354</v>
@@ -3500,7 +5704,7 @@
         <v>5512796</v>
       </c>
       <c r="H19" s="11" t="n">
-        <v>0.4816</v>
+        <v>0.5716</v>
       </c>
       <c r="I19" s="11" t="n">
         <v>0.3486</v>
@@ -3543,7 +5747,7 @@
         <v>9370589</v>
       </c>
       <c r="H20" s="11" t="n">
-        <v>0.4816</v>
+        <v>0.6038</v>
       </c>
       <c r="I20" s="11" t="n">
         <v>0.344</v>
@@ -3586,7 +5790,7 @@
         <v>12363246</v>
       </c>
       <c r="H21" s="11" t="n">
-        <v>0.4816</v>
+        <v>0.6002000000000001</v>
       </c>
       <c r="I21" s="11" t="n">
         <v>0.3256</v>
@@ -3629,7 +5833,7 @@
         <v>9845111</v>
       </c>
       <c r="H22" s="11" t="n">
-        <v>0.4816</v>
+        <v>0.5922999999999999</v>
       </c>
       <c r="I22" s="11" t="n">
         <v>0.2813</v>
@@ -3672,7 +5876,7 @@
         <v>9562382</v>
       </c>
       <c r="H23" s="11" t="n">
-        <v>0.4816</v>
+        <v>0.6049</v>
       </c>
       <c r="I23" s="11" t="n">
         <v>0.3146</v>
@@ -3715,7 +5919,7 @@
         <v>16160186</v>
       </c>
       <c r="H24" s="11" t="n">
-        <v>0.4816</v>
+        <v>0.5939</v>
       </c>
       <c r="I24" s="11" t="n">
         <v>0.3856</v>
@@ -3758,7 +5962,7 @@
         <v>15568073</v>
       </c>
       <c r="H25" s="11" t="n">
-        <v>0.4816</v>
+        <v>0.6161</v>
       </c>
       <c r="I25" s="11" t="n">
         <v>0.3765</v>
@@ -3801,7 +6005,7 @@
         <v>7232750</v>
       </c>
       <c r="H26" s="11" t="n">
-        <v>0.4816</v>
+        <v>0.6198</v>
       </c>
       <c r="I26" s="11" t="n">
         <v>0.3647</v>
@@ -3844,7 +6048,7 @@
         <v>11383349</v>
       </c>
       <c r="H27" s="11" t="n">
-        <v>0.4816</v>
+        <v>0.6343</v>
       </c>
       <c r="I27" s="11" t="n">
         <v>0.3861</v>
@@ -3887,7 +6091,7 @@
         <v>13381960</v>
       </c>
       <c r="H28" s="11" t="n">
-        <v>0.4816</v>
+        <v>0.6183</v>
       </c>
       <c r="I28" s="11" t="n">
         <v>0.3211</v>
@@ -3930,7 +6134,7 @@
         <v>9008514</v>
       </c>
       <c r="H29" s="11" t="n">
-        <v>0.4816</v>
+        <v>0.6143999999999999</v>
       </c>
       <c r="I29" s="11" t="n">
         <v>0.3433</v>
@@ -3973,7 +6177,7 @@
         <v>7506867</v>
       </c>
       <c r="H30" s="11" t="n">
-        <v>0.4816</v>
+        <v>0.6175</v>
       </c>
       <c r="I30" s="11" t="n">
         <v>0.3898</v>
@@ -4016,7 +6220,7 @@
         <v>11160815</v>
       </c>
       <c r="H31" s="11" t="n">
-        <v>0.4816</v>
+        <v>0.6455</v>
       </c>
       <c r="I31" s="11" t="n">
         <v>0.3762</v>
@@ -4059,7 +6263,7 @@
         <v>12728635</v>
       </c>
       <c r="H32" s="11" t="n">
-        <v>0.4816</v>
+        <v>0.6204</v>
       </c>
       <c r="I32" s="11" t="n">
         <v>0.3658</v>
@@ -4102,7 +6306,7 @@
         <v>9774024</v>
       </c>
       <c r="H33" s="11" t="n">
-        <v>0.4816</v>
+        <v>0.6148</v>
       </c>
       <c r="I33" s="11" t="n">
         <v>0.4301</v>
@@ -4145,7 +6349,7 @@
         <v>12995978</v>
       </c>
       <c r="H34" s="11" t="n">
-        <v>0.4816</v>
+        <v>0.6411</v>
       </c>
       <c r="I34" s="11" t="n">
         <v>0.474</v>
@@ -4188,7 +6392,7 @@
         <v>10158090</v>
       </c>
       <c r="H35" s="11" t="n">
-        <v>0.4816</v>
+        <v>0.6381</v>
       </c>
       <c r="I35" s="11" t="n">
         <v>0.4234000000000001</v>
@@ -4231,7 +6435,7 @@
         <v>8471978</v>
       </c>
       <c r="H36" s="11" t="n">
-        <v>0.4816</v>
+        <v>0.6048</v>
       </c>
       <c r="I36" s="11" t="n">
         <v>0.3584000000000001</v>
@@ -4256,7 +6460,7 @@
         </is>
       </c>
       <c r="B37" s="6" t="n">
-        <v>828788847.17</v>
+        <v>733490124.87</v>
       </c>
       <c r="C37" s="6" t="n">
         <v>12490106.43</v>
@@ -4274,7 +6478,7 @@
         <v>11868618</v>
       </c>
       <c r="H37" s="11" t="n">
-        <v>0.4816</v>
+        <v>0.6257</v>
       </c>
       <c r="I37" s="11" t="n">
         <v>0.3806</v>
@@ -4298,9 +6502,7 @@
           <t>2026-09-05</t>
         </is>
       </c>
-      <c r="B38" s="6" t="n">
-        <v>1128108281.21</v>
-      </c>
+      <c r="B38" s="6" t="n"/>
       <c r="C38" s="6" t="n">
         <v>18169819.03</v>
       </c>
@@ -4316,9 +6518,7 @@
       <c r="G38" s="6" t="n">
         <v>10824093</v>
       </c>
-      <c r="H38" s="11" t="n">
-        <v>0.4816</v>
-      </c>
+      <c r="H38" s="11" t="n"/>
       <c r="I38" s="11" t="n">
         <v>0.3624</v>
       </c>
@@ -4335,15 +6535,54 @@
         <v>0.3572</v>
       </c>
     </row>
-    <row r="40">
-      <c r="A40" s="12" t="inlineStr">
-        <is>
-          <t>Kalshi = its KXMVE multi-event parlay engine (leg-checked ~100% sports legs despite the 'cross-category' name), from a ~3M-trade sample of the public feed scaled to the daily total. Its % is of its WHOLE-EXCHANGE volume (matching its main column) - ~48% by contracts / ~11% by $. Sample-based, so it moves less day to day; not folded into the Daily tab's blended Combo %. Rothera runs no on-exchange parlay product and is omitted here.</t>
+    <row r="39">
+      <c r="A39" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="B39" s="6" t="n"/>
+      <c r="C39" s="6" t="n">
+        <v>10625376.42</v>
+      </c>
+      <c r="D39" s="6" t="n">
+        <v>15329162</v>
+      </c>
+      <c r="E39" s="6" t="n">
+        <v>40590069.68</v>
+      </c>
+      <c r="F39" s="6" t="n">
+        <v>13770949.4</v>
+      </c>
+      <c r="G39" s="6" t="n">
+        <v>12319196</v>
+      </c>
+      <c r="H39" s="11" t="n"/>
+      <c r="I39" s="11" t="n">
+        <v>0.3315</v>
+      </c>
+      <c r="J39" s="11" t="n">
+        <v>0.4267</v>
+      </c>
+      <c r="K39" s="11" t="n">
+        <v>0.3089</v>
+      </c>
+      <c r="L39" s="11" t="n">
+        <v>0.6354</v>
+      </c>
+      <c r="M39" s="11" t="n">
+        <v>0.3801</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="12" t="inlineStr">
+        <is>
+          <t>Combo % = parlay volume / that venue's sports book. Kalshi's parlay is its KXMVE multi-event engine (leg-checked ~100% sports legs despite the 'cross-category' name), from a ~3M-trade sample scaled to the daily total; ~62% of Kalshi's sports book by contracts, ~18% by $ (parlay legs are many and cheap). Not folded into the Sports tab's blended Combo % (sample-based, moves less day to day). Rothera runs no on-exchange parlay product.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A2:M38"/>
+  <autoFilter ref="A2:M39"/>
   <mergeCells count="2">
     <mergeCell ref="H1:M1"/>
     <mergeCell ref="B1:G1"/>
@@ -4352,29 +6591,29 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A30"/>
+  <dimension ref="A1:A23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="92" customWidth="1" min="1" max="1"/>
+    <col width="95" customWidth="1" min="1" max="1"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="13" t="inlineStr">
         <is>
-          <t>Sports prediction-market volume - daily</t>
+          <t>US prediction-market volume - daily, 7 regulated exchanges</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Generated 2026-09-06 from unified_sports_volume.csv</t>
+          <t>Generated 2026-09-07. Full detail: VOLUME_METHODOLOGY.md</t>
         </is>
       </c>
     </row>
@@ -4384,101 +6623,97 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>One comparable metric for all seven venues: contracts traded, one-sided</t>
+          <t>One comparable metric: contracts traded, one-sided (a buy matched with a</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>(a buy matched with a sell counts once), each contract a $1-max-payout</t>
+          <t>sell counts once), each a $1-max-payout instrument. 'Notional $' re-weights</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>instrument. 'Notional $' re-weights each contract by its traded price</t>
+          <t>each contract by its traded price (~ the dollars that changed hands).</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>(~ the dollars that changed hands, roughly 1/3 of the contract count).</t>
-        </is>
-      </c>
+      <c r="A7" t="inlineStr"/>
     </row>
     <row r="8">
-      <c r="A8" t="inlineStr"/>
+      <c r="A8" s="13" t="inlineStr">
+        <is>
+          <t>TAB 'Sports volume'  - each venue's sports book only. Apples-to-apples on sports.</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Kalshi   = WHOLE exchange, every category (daily total from DeFi Rate; the</t>
+          <t xml:space="preserve">  Kalshi = single-leg sports + its sports parlay engine.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t xml:space="preserve">           last ~2-3 days are projected - see the 'source' column upstream).</t>
+          <t xml:space="preserve">  Polymarket US / Crypto.com / Rothera = sports filtered out of a wider book.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Polymarket US = sports, symbol-prefix filtered.</t>
+          <t xml:space="preserve">  Novig / DKeX / UDX = sports-only exchanges (their sports IS their whole book).</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>Novig / DKeX / UDX = 100% sports, from their CFTC Part-16 daily reports.</t>
-        </is>
-      </c>
+      <c r="A12" t="inlineStr"/>
     </row>
     <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>Crypto.com = Nadex / CDNA 'EVENTS' book - Crypto.com's own prediction market</t>
+      <c r="A13" s="13" t="inlineStr">
+        <is>
+          <t>TAB 'Total exchange'  - each venue's WHOLE book, every category (sports, crypto,</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t xml:space="preserve">           plus FanDuel Predicts (all its sports flow clears there), minus a</t>
+          <t xml:space="preserve">  politics, economics, ...). Apples-to-apples on total platform activity.</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t xml:space="preserve">           ~0.2% non-sports tail. Notional $ uses the cross-venue avg price.</t>
+          <t xml:space="preserve">  Kalshi total from DeFi Rate (last ~2 days projected). Polymarket = all QCX.</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Rothera  = the CFTC exchange behind Robinhood's prediction market (Part-16</t>
+          <t xml:space="preserve">  Crypto.com = the whole Nadex/CDNA book (events + fx/commodity/crypto binaries).</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t xml:space="preserve">           daily report). Prefix-filtered to sports (MLB-heavy); a small</t>
+          <t xml:space="preserve">  Rothera = sports + its US-macro / elections markets.</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t xml:space="preserve">           US-macro / elections tail is dropped.</t>
+          <t xml:space="preserve">  Novig / DKeX / UDX total == their sports figure (sports-only exchanges).</t>
         </is>
       </c>
     </row>
@@ -4486,75 +6721,26 @@
       <c r="A19" t="inlineStr"/>
     </row>
     <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>Combos: tracked per-venue on the 'Parlay share' tab. Novig / DKeX /</t>
+      <c r="A20" s="13" t="inlineStr">
+        <is>
+          <t>TAB 'Parlay share'  - per-venue combo/parlay volume and % of that venue's sports book.</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t xml:space="preserve">        Polymarket US / UDX / Crypto.com from their combo product line</t>
-        </is>
-      </c>
+      <c r="A21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t xml:space="preserve">        (% of that venue's book). Kalshi = its KXMVE multi-event parlay</t>
+          <t>UDX and Crypto.com have no usable price column - their Notional $ is estimated</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t xml:space="preserve">        engine (leg-checked ~100% sports legs), from a ~3M-trade sample</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" t="inlineStr">
-        <is>
-          <t xml:space="preserve">        scaled to the daily total, as a % of its WHOLE-EXCHANGE volume</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" t="inlineStr">
-        <is>
-          <t xml:space="preserve">        (matching its main column) - ~48% by contracts / ~11% by $. The</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" t="inlineStr">
-        <is>
-          <t xml:space="preserve">        Daily tab's blended Combo % is the five report-based venues only;</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" t="inlineStr">
-        <is>
-          <t xml:space="preserve">        Rothera has no on-exchange parlay product.</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" t="inlineStr"/>
-    </row>
-    <row r="29">
-      <c r="A29" t="inlineStr">
-        <is>
-          <t>All seven US CFTC sports-prediction venues are covered.</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" t="inlineStr">
-        <is>
-          <t>Full detail: VOLUME_METHODOLOGY.md</t>
+          <t>with the day's contract-weighted average price across the venues that report one.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Fix: remove conflict markers from bd61463, harden CI commit step
bd61463's rebase left merge-conflict markers in 12 generated CSVs, which
crashed the pipeline. Restored clean data, regenerated the schema-changed
files. The workflow now aborts its commit on a rebase conflict instead of
ever pushing markers.
</commit_message>
<xml_diff>
--- a/unified_sports_volume.xlsx
+++ b/unified_sports_volume.xlsx
@@ -13,9 +13,9 @@
     <sheet name="Notes" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Sports volume'!$A$2:$R$39</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Total exchange'!$A$2:$Q$39</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Parlay share'!$A$2:$M$39</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Sports volume'!$A$2:$R$40</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Total exchange'!$A$2:$Q$40</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Parlay share'!$A$2:$M$40</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -479,7 +479,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R39"/>
+  <dimension ref="A1:R40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -618,7 +618,7 @@
         </is>
       </c>
       <c r="B3" s="5" t="n">
-        <v>1226348301.09</v>
+        <v>1226349065.69</v>
       </c>
       <c r="C3" s="6" t="n">
         <v>133399888.66</v>
@@ -637,10 +637,10 @@
         <v>4370899</v>
       </c>
       <c r="I3" s="7" t="n">
-        <v>1404310395.67</v>
+        <v>1404311160.27</v>
       </c>
       <c r="J3" s="8" t="n">
-        <v>290712233.4</v>
+        <v>290712357.9</v>
       </c>
       <c r="K3" s="9" t="n">
         <v>50986272.22</v>
@@ -650,16 +650,16 @@
         <v>436176.76</v>
       </c>
       <c r="N3" s="9" t="n">
-        <v>524812.1800000001</v>
+        <v>524812.08</v>
       </c>
       <c r="O3" s="9" t="n">
-        <v>9360273.49</v>
+        <v>9360271.630000001</v>
       </c>
       <c r="P3" s="9" t="n">
         <v>2035457.65</v>
       </c>
       <c r="Q3" s="9" t="n">
-        <v>354055225.7</v>
+        <v>354055348.24</v>
       </c>
       <c r="R3" s="10" t="n">
         <v>0.08714584215412201</v>
@@ -672,7 +672,7 @@
         </is>
       </c>
       <c r="B4" s="5" t="n">
-        <v>1019790521.49</v>
+        <v>1019791784.21</v>
       </c>
       <c r="C4" s="6" t="n">
         <v>134065934.54</v>
@@ -691,10 +691,10 @@
         <v>7690938</v>
       </c>
       <c r="I4" s="7" t="n">
-        <v>1203195431</v>
+        <v>1203196693.72</v>
       </c>
       <c r="J4" s="8" t="n">
-        <v>223745816.63</v>
+        <v>223745991.8</v>
       </c>
       <c r="K4" s="9" t="n">
         <v>51144509.72</v>
@@ -704,16 +704,16 @@
         <v>484971.88</v>
       </c>
       <c r="N4" s="9" t="n">
-        <v>516298.92</v>
+        <v>516298.68</v>
       </c>
       <c r="O4" s="9" t="n">
-        <v>9237390.460000001</v>
+        <v>9237386.220000001</v>
       </c>
       <c r="P4" s="9" t="n">
         <v>3928624.18</v>
       </c>
       <c r="Q4" s="9" t="n">
-        <v>289057611.79</v>
+        <v>289057782.49</v>
       </c>
       <c r="R4" s="10" t="n">
         <v>0.07635377691307524</v>
@@ -726,7 +726,7 @@
         </is>
       </c>
       <c r="B5" s="5" t="n">
-        <v>766399762</v>
+        <v>766400758.2</v>
       </c>
       <c r="C5" s="6" t="n">
         <v>85344135.09999999</v>
@@ -745,10 +745,10 @@
         <v>9061437</v>
       </c>
       <c r="I5" s="7" t="n">
-        <v>882442309.04</v>
+        <v>882443305.24</v>
       </c>
       <c r="J5" s="8" t="n">
-        <v>197400001.9</v>
+        <v>197400445.99</v>
       </c>
       <c r="K5" s="9" t="n">
         <v>31777180.84</v>
@@ -758,16 +758,16 @@
         <v>165403.4</v>
       </c>
       <c r="N5" s="9" t="n">
-        <v>374709.28</v>
+        <v>374709.56</v>
       </c>
       <c r="O5" s="9" t="n">
-        <v>5399343.04</v>
+        <v>5399347.05</v>
       </c>
       <c r="P5" s="9" t="n">
         <v>4372698.14</v>
       </c>
       <c r="Q5" s="9" t="n">
-        <v>239489336.6</v>
+        <v>239489784.98</v>
       </c>
       <c r="R5" s="10" t="n">
         <v>0.05231046649197771</v>
@@ -780,7 +780,7 @@
         </is>
       </c>
       <c r="B6" s="5" t="n">
-        <v>983748421.3200001</v>
+        <v>983749291.22</v>
       </c>
       <c r="C6" s="6" t="n">
         <v>120394335.41</v>
@@ -801,10 +801,10 @@
         <v>16424385</v>
       </c>
       <c r="I6" s="7" t="n">
-        <v>1168386570.34</v>
+        <v>1168387440.24</v>
       </c>
       <c r="J6" s="8" t="n">
-        <v>236058435.39</v>
+        <v>236058651.18</v>
       </c>
       <c r="K6" s="9" t="n">
         <v>47471997.74</v>
@@ -816,16 +816,16 @@
         <v>222905.14</v>
       </c>
       <c r="N6" s="9" t="n">
-        <v>324586.19</v>
+        <v>324586.17</v>
       </c>
       <c r="O6" s="9" t="n">
-        <v>7358489.61</v>
+        <v>7358489.32</v>
       </c>
       <c r="P6" s="9" t="n">
         <v>8062430.32</v>
       </c>
       <c r="Q6" s="9" t="n">
-        <v>305855095.76</v>
+        <v>305855311.24</v>
       </c>
       <c r="R6" s="10" t="n">
         <v>0.1040882840699126</v>
@@ -838,7 +838,7 @@
         </is>
       </c>
       <c r="B7" s="5" t="n">
-        <v>1097580318.95</v>
+        <v>1097584373.29</v>
       </c>
       <c r="C7" s="6" t="n">
         <v>125055737.8</v>
@@ -859,10 +859,10 @@
         <v>25367258</v>
       </c>
       <c r="I7" s="7" t="n">
-        <v>1302660356.53</v>
+        <v>1302664410.87</v>
       </c>
       <c r="J7" s="8" t="n">
-        <v>250948122.31</v>
+        <v>250949776.33</v>
       </c>
       <c r="K7" s="9" t="n">
         <v>47948549.82</v>
@@ -874,16 +874,16 @@
         <v>292548.17</v>
       </c>
       <c r="N7" s="9" t="n">
-        <v>709925.6800000001</v>
+        <v>709927.08</v>
       </c>
       <c r="O7" s="9" t="n">
-        <v>7693337.29</v>
+        <v>7693352.53</v>
       </c>
       <c r="P7" s="9" t="n">
         <v>12897725.83</v>
       </c>
       <c r="Q7" s="9" t="n">
-        <v>328052116.54</v>
+        <v>328053787.2</v>
       </c>
       <c r="R7" s="10" t="n">
         <v>0.1036604405692761</v>
@@ -896,7 +896,7 @@
         </is>
       </c>
       <c r="B8" s="5" t="n">
-        <v>1011514178.87</v>
+        <v>1011515724.09</v>
       </c>
       <c r="C8" s="6" t="n">
         <v>141146850.05</v>
@@ -917,10 +917,10 @@
         <v>23442413</v>
       </c>
       <c r="I8" s="7" t="n">
-        <v>1233687298.38</v>
+        <v>1233688843.6</v>
       </c>
       <c r="J8" s="8" t="n">
-        <v>229522489.57</v>
+        <v>229523163.57</v>
       </c>
       <c r="K8" s="9" t="n">
         <v>50551741.94</v>
@@ -932,16 +932,16 @@
         <v>314539.43</v>
       </c>
       <c r="N8" s="9" t="n">
-        <v>1255741.5</v>
+        <v>1255742.7</v>
       </c>
       <c r="O8" s="9" t="n">
-        <v>8409716.380000001</v>
+        <v>8409724.43</v>
       </c>
       <c r="P8" s="9" t="n">
         <v>11914017.45</v>
       </c>
       <c r="Q8" s="9" t="n">
-        <v>309197404.1</v>
+        <v>309198087.35</v>
       </c>
       <c r="R8" s="10" t="n">
         <v>0.09320593928966855</v>
@@ -954,7 +954,7 @@
         </is>
       </c>
       <c r="B9" s="5" t="n">
-        <v>961933487.02</v>
+        <v>961934760.5599999</v>
       </c>
       <c r="C9" s="6" t="n">
         <v>117925601.54</v>
@@ -975,10 +975,10 @@
         <v>18014225</v>
       </c>
       <c r="I9" s="7" t="n">
-        <v>1145540648.56</v>
+        <v>1145541922.1</v>
       </c>
       <c r="J9" s="8" t="n">
-        <v>214888229.88</v>
+        <v>214888631.7</v>
       </c>
       <c r="K9" s="9" t="n">
         <v>44939973.52</v>
@@ -990,16 +990,16 @@
         <v>280061.26</v>
       </c>
       <c r="N9" s="9" t="n">
-        <v>814778.05</v>
+        <v>814778.3199999999</v>
       </c>
       <c r="O9" s="9" t="n">
-        <v>6850540.39</v>
+        <v>6850542.63</v>
       </c>
       <c r="P9" s="9" t="n">
         <v>8768403.85</v>
       </c>
       <c r="Q9" s="9" t="n">
-        <v>281205393.52</v>
+        <v>281205797.84</v>
       </c>
       <c r="R9" s="10" t="n">
         <v>0.100308786205459</v>
@@ -1012,7 +1012,7 @@
         </is>
       </c>
       <c r="B10" s="5" t="n">
-        <v>1073038713.76</v>
+        <v>1073041912.66</v>
       </c>
       <c r="C10" s="6" t="n">
         <v>119094679.49</v>
@@ -1033,10 +1033,10 @@
         <v>23158725</v>
       </c>
       <c r="I10" s="7" t="n">
-        <v>1277704611.24</v>
+        <v>1277707810.14</v>
       </c>
       <c r="J10" s="8" t="n">
-        <v>240123237.17</v>
+        <v>240123982.18</v>
       </c>
       <c r="K10" s="9" t="n">
         <v>44015511.37</v>
@@ -1048,16 +1048,16 @@
         <v>545929.65</v>
       </c>
       <c r="N10" s="9" t="n">
-        <v>2353400.13</v>
+        <v>2353399.81</v>
       </c>
       <c r="O10" s="9" t="n">
-        <v>7569915.52</v>
+        <v>7569914.51</v>
       </c>
       <c r="P10" s="9" t="n">
         <v>11672366.2</v>
       </c>
       <c r="Q10" s="9" t="n">
-        <v>313747030.7</v>
+        <v>313747774.39</v>
       </c>
       <c r="R10" s="10" t="n">
         <v>0.1305164739611011</v>
@@ -1070,7 +1070,7 @@
         </is>
       </c>
       <c r="B11" s="5" t="n">
-        <v>960754930.92</v>
+        <v>960755772.36</v>
       </c>
       <c r="C11" s="6" t="n">
         <v>126075255.12</v>
@@ -1091,10 +1091,10 @@
         <v>33913543</v>
       </c>
       <c r="I11" s="7" t="n">
-        <v>1185428248.04</v>
+        <v>1185429089.48</v>
       </c>
       <c r="J11" s="8" t="n">
-        <v>212543726.02</v>
+        <v>212543924.4</v>
       </c>
       <c r="K11" s="9" t="n">
         <v>48533344.05</v>
@@ -1106,16 +1106,16 @@
         <v>391311.2</v>
       </c>
       <c r="N11" s="9" t="n">
-        <v>2490144.51</v>
+        <v>2490144.41</v>
       </c>
       <c r="O11" s="9" t="n">
-        <v>8929257.99</v>
+        <v>8929257.619999999</v>
       </c>
       <c r="P11" s="9" t="n">
         <v>17131109.38</v>
       </c>
       <c r="Q11" s="9" t="n">
-        <v>296178469.23</v>
+        <v>296178667.13</v>
       </c>
       <c r="R11" s="10" t="n">
         <v>0.1174147553025735</v>
@@ -1128,7 +1128,7 @@
         </is>
       </c>
       <c r="B12" s="5" t="n">
-        <v>686488587.74</v>
+        <v>686491037.87</v>
       </c>
       <c r="C12" s="6" t="n">
         <v>76773291.01000001</v>
@@ -1149,10 +1149,10 @@
         <v>11323712</v>
       </c>
       <c r="I12" s="7" t="n">
-        <v>813400278.77</v>
+        <v>813402728.9</v>
       </c>
       <c r="J12" s="8" t="n">
-        <v>150986874.89</v>
+        <v>150987576.69</v>
       </c>
       <c r="K12" s="9" t="n">
         <v>28141958.88</v>
@@ -1164,16 +1164,16 @@
         <v>146839.93</v>
       </c>
       <c r="N12" s="9" t="n">
-        <v>1897060.47</v>
+        <v>1897061.57</v>
       </c>
       <c r="O12" s="9" t="n">
-        <v>3485519.72</v>
+        <v>3485521.74</v>
       </c>
       <c r="P12" s="9" t="n">
         <v>5809820.01</v>
       </c>
       <c r="Q12" s="9" t="n">
-        <v>196251414.98</v>
+        <v>196252119.9</v>
       </c>
       <c r="R12" s="10" t="n">
         <v>0.1320471995718654</v>
@@ -1186,7 +1186,7 @@
         </is>
       </c>
       <c r="B13" s="5" t="n">
-        <v>970895177.89</v>
+        <v>970898610.01</v>
       </c>
       <c r="C13" s="6" t="n">
         <v>86060025.34</v>
@@ -1207,10 +1207,10 @@
         <v>19659153</v>
       </c>
       <c r="I13" s="7" t="n">
-        <v>1130451832.13</v>
+        <v>1130455264.25</v>
       </c>
       <c r="J13" s="8" t="n">
-        <v>227536176.85</v>
+        <v>227537789.85</v>
       </c>
       <c r="K13" s="9" t="n">
         <v>32573678.23</v>
@@ -1222,16 +1222,16 @@
         <v>342568.77</v>
       </c>
       <c r="N13" s="9" t="n">
-        <v>2642012.55</v>
+        <v>2642019.6</v>
       </c>
       <c r="O13" s="9" t="n">
-        <v>5513093.35</v>
+        <v>5513108.06</v>
       </c>
       <c r="P13" s="9" t="n">
         <v>9689300.880000001</v>
       </c>
       <c r="Q13" s="9" t="n">
-        <v>286533831.19</v>
+        <v>286535465.96</v>
       </c>
       <c r="R13" s="10" t="n">
         <v>0.1581581529884586</v>
@@ -1244,7 +1244,7 @@
         </is>
       </c>
       <c r="B14" s="5" t="n">
-        <v>1042720983.61</v>
+        <v>1042722691.8</v>
       </c>
       <c r="C14" s="6" t="n">
         <v>114182203.82</v>
@@ -1265,10 +1265,10 @@
         <v>23900271</v>
       </c>
       <c r="I14" s="7" t="n">
-        <v>1244205173.68</v>
+        <v>1244206881.87</v>
       </c>
       <c r="J14" s="8" t="n">
-        <v>230879117.13</v>
+        <v>230880141.16</v>
       </c>
       <c r="K14" s="9" t="n">
         <v>44020201.24</v>
@@ -1280,16 +1280,16 @@
         <v>463531.04</v>
       </c>
       <c r="N14" s="9" t="n">
-        <v>2865649.45</v>
+        <v>2865655.3</v>
       </c>
       <c r="O14" s="9" t="n">
-        <v>7026032.49</v>
+        <v>7026046.84</v>
       </c>
       <c r="P14" s="9" t="n">
         <v>11689925.33</v>
       </c>
       <c r="Q14" s="9" t="n">
-        <v>305683870.5</v>
+        <v>305684914.74</v>
       </c>
       <c r="R14" s="10" t="n">
         <v>0.1369006174109096</v>
@@ -1302,7 +1302,7 @@
         </is>
       </c>
       <c r="B15" s="5" t="n">
-        <v>1046511668.87</v>
+        <v>1046512903.29</v>
       </c>
       <c r="C15" s="6" t="n">
         <v>130618679.53</v>
@@ -1323,10 +1323,10 @@
         <v>24114127</v>
       </c>
       <c r="I15" s="7" t="n">
-        <v>1268558768.68</v>
+        <v>1268560003.1</v>
       </c>
       <c r="J15" s="8" t="n">
-        <v>238375725.51</v>
+        <v>238375967.85</v>
       </c>
       <c r="K15" s="9" t="n">
         <v>47519466.33</v>
@@ -1338,16 +1338,16 @@
         <v>401500.01</v>
       </c>
       <c r="N15" s="9" t="n">
-        <v>3737679.55</v>
+        <v>3737678.75</v>
       </c>
       <c r="O15" s="9" t="n">
-        <v>7838233.09</v>
+        <v>7838231.42</v>
       </c>
       <c r="P15" s="9" t="n">
         <v>11390787.92</v>
       </c>
       <c r="Q15" s="9" t="n">
-        <v>315842374.95</v>
+        <v>315842614.82</v>
       </c>
       <c r="R15" s="10" t="n">
         <v>0.1338434618903201</v>
@@ -1360,7 +1360,7 @@
         </is>
       </c>
       <c r="B16" s="5" t="n">
-        <v>1026507894.75</v>
+        <v>1026509230.11</v>
       </c>
       <c r="C16" s="6" t="n">
         <v>122512075.89</v>
@@ -1381,10 +1381,10 @@
         <v>13420824</v>
       </c>
       <c r="I16" s="7" t="n">
-        <v>1228651773.78</v>
+        <v>1228653109.14</v>
       </c>
       <c r="J16" s="8" t="n">
-        <v>246149823.25</v>
+        <v>246150132.87</v>
       </c>
       <c r="K16" s="9" t="n">
         <v>44967846.15</v>
@@ -1396,16 +1396,16 @@
         <v>598777.14</v>
       </c>
       <c r="N16" s="9" t="n">
-        <v>3558650.45</v>
+        <v>3558650.06</v>
       </c>
       <c r="O16" s="9" t="n">
-        <v>7537326.75</v>
+        <v>7537325.92</v>
       </c>
       <c r="P16" s="9" t="n">
         <v>5908662.92</v>
       </c>
       <c r="Q16" s="9" t="n">
-        <v>315569854.61</v>
+        <v>315570163.01</v>
       </c>
       <c r="R16" s="10" t="n">
         <v>0.1467243571212392</v>
@@ -1418,7 +1418,7 @@
         </is>
       </c>
       <c r="B17" s="5" t="n">
-        <v>1275197725.87</v>
+        <v>1275202312.3</v>
       </c>
       <c r="C17" s="6" t="n">
         <v>135215397.14</v>
@@ -1439,10 +1439,10 @@
         <v>23624339</v>
       </c>
       <c r="I17" s="7" t="n">
-        <v>1517919203.12</v>
+        <v>1517923789.55</v>
       </c>
       <c r="J17" s="8" t="n">
-        <v>295667968.4</v>
+        <v>295668395.47</v>
       </c>
       <c r="K17" s="9" t="n">
         <v>48968794.7</v>
@@ -1454,16 +1454,16 @@
         <v>899431.51</v>
       </c>
       <c r="N17" s="9" t="n">
-        <v>4271142.9</v>
+        <v>4271134.51</v>
       </c>
       <c r="O17" s="9" t="n">
-        <v>9581206.310000001</v>
+        <v>9581187.48</v>
       </c>
       <c r="P17" s="9" t="n">
         <v>11142968.25</v>
       </c>
       <c r="Q17" s="9" t="n">
-        <v>378764313.5</v>
+        <v>378764713.34</v>
       </c>
       <c r="R17" s="10" t="n">
         <v>0.1671310595982739</v>
@@ -1476,7 +1476,7 @@
         </is>
       </c>
       <c r="B18" s="5" t="n">
-        <v>1123162110.77</v>
+        <v>1123165604.25</v>
       </c>
       <c r="C18" s="6" t="n">
         <v>146617403.12</v>
@@ -1497,10 +1497,10 @@
         <v>24327302</v>
       </c>
       <c r="I18" s="7" t="n">
-        <v>1375337272.1</v>
+        <v>1375340765.58</v>
       </c>
       <c r="J18" s="8" t="n">
-        <v>251871816.77</v>
+        <v>251873332.44</v>
       </c>
       <c r="K18" s="9" t="n">
         <v>56978627.74</v>
@@ -1512,16 +1512,16 @@
         <v>644960.33</v>
       </c>
       <c r="N18" s="9" t="n">
-        <v>3520463.22</v>
+        <v>3520470.22</v>
       </c>
       <c r="O18" s="9" t="n">
-        <v>11255639.31</v>
+        <v>11255661.71</v>
       </c>
       <c r="P18" s="9" t="n">
         <v>11565704.7</v>
       </c>
       <c r="Q18" s="9" t="n">
-        <v>341090876.14</v>
+        <v>341092421.21</v>
       </c>
       <c r="R18" s="10" t="n">
         <v>0.1404248555660547</v>
@@ -1534,7 +1534,7 @@
         </is>
       </c>
       <c r="B19" s="5" t="n">
-        <v>780468036.02</v>
+        <v>780472551.89</v>
       </c>
       <c r="C19" s="6" t="n">
         <v>100434174.96</v>
@@ -1555,10 +1555,10 @@
         <v>11675481</v>
       </c>
       <c r="I19" s="7" t="n">
-        <v>941884881.55</v>
+        <v>941889397.42</v>
       </c>
       <c r="J19" s="8" t="n">
-        <v>182876983.93</v>
+        <v>182878296.39</v>
       </c>
       <c r="K19" s="9" t="n">
         <v>36933011.94</v>
@@ -1570,16 +1570,16 @@
         <v>587784.12</v>
       </c>
       <c r="N19" s="9" t="n">
-        <v>2893225.33</v>
+        <v>2893227.32</v>
       </c>
       <c r="O19" s="9" t="n">
-        <v>4978949.19</v>
+        <v>4978952.62</v>
       </c>
       <c r="P19" s="9" t="n">
         <v>5508381.8</v>
       </c>
       <c r="Q19" s="9" t="n">
-        <v>240361001.38</v>
+        <v>240362319.26</v>
       </c>
       <c r="R19" s="10" t="n">
         <v>0.1248997633733931</v>
@@ -1592,7 +1592,7 @@
         </is>
       </c>
       <c r="B20" s="5" t="n">
-        <v>925190752.63</v>
+        <v>925196477.27</v>
       </c>
       <c r="C20" s="6" t="n">
         <v>104121932.82</v>
@@ -1613,10 +1613,10 @@
         <v>14628870</v>
       </c>
       <c r="I20" s="7" t="n">
-        <v>1103194136.45</v>
+        <v>1103199861.09</v>
       </c>
       <c r="J20" s="8" t="n">
-        <v>208930058.54</v>
+        <v>208931948.3</v>
       </c>
       <c r="K20" s="9" t="n">
         <v>38002578.37</v>
@@ -1628,16 +1628,16 @@
         <v>262338.04</v>
       </c>
       <c r="N20" s="9" t="n">
-        <v>3099127.65</v>
+        <v>3099133.4</v>
       </c>
       <c r="O20" s="9" t="n">
-        <v>6218628.53</v>
+        <v>6218640.06</v>
       </c>
       <c r="P20" s="9" t="n">
         <v>6862320.27</v>
       </c>
       <c r="Q20" s="9" t="n">
-        <v>270748324.73</v>
+        <v>270750231.77</v>
       </c>
       <c r="R20" s="10" t="n">
         <v>0.178213812300984</v>
@@ -1650,7 +1650,7 @@
         </is>
       </c>
       <c r="B21" s="5" t="n">
-        <v>1099235509.23</v>
+        <v>1099239543.2</v>
       </c>
       <c r="C21" s="6" t="n">
         <v>122677612.96</v>
@@ -1671,10 +1671,10 @@
         <v>21296436</v>
       </c>
       <c r="I21" s="7" t="n">
-        <v>1314535803.05</v>
+        <v>1314539837.02</v>
       </c>
       <c r="J21" s="8" t="n">
-        <v>244612818.63</v>
+        <v>244614998.21</v>
       </c>
       <c r="K21" s="9" t="n">
         <v>44708007.56</v>
@@ -1686,16 +1686,16 @@
         <v>691813.04</v>
       </c>
       <c r="N21" s="9" t="n">
-        <v>3671151</v>
+        <v>3671165.29</v>
       </c>
       <c r="O21" s="9" t="n">
-        <v>7710470.83</v>
+        <v>7710500.84</v>
       </c>
       <c r="P21" s="9" t="n">
         <v>10373288.39</v>
       </c>
       <c r="Q21" s="9" t="n">
-        <v>319466861.16</v>
+        <v>319469085.04</v>
       </c>
       <c r="R21" s="10" t="n">
         <v>0.2003579150386557</v>
@@ -1708,7 +1708,7 @@
         </is>
       </c>
       <c r="B22" s="5" t="n">
-        <v>967567863.75</v>
+        <v>967573101.1799999</v>
       </c>
       <c r="C22" s="6" t="n">
         <v>132905659.86</v>
@@ -1729,10 +1729,10 @@
         <v>24665675</v>
       </c>
       <c r="I22" s="7" t="n">
-        <v>1190888869.33</v>
+        <v>1190894106.76</v>
       </c>
       <c r="J22" s="8" t="n">
-        <v>210526920.69</v>
+        <v>210527933.59</v>
       </c>
       <c r="K22" s="9" t="n">
         <v>44439935.08</v>
@@ -1744,16 +1744,16 @@
         <v>426029.96</v>
       </c>
       <c r="N22" s="9" t="n">
-        <v>3281796.18</v>
+        <v>3281793.35</v>
       </c>
       <c r="O22" s="9" t="n">
-        <v>7536291.6</v>
+        <v>7536285.11</v>
       </c>
       <c r="P22" s="9" t="n">
         <v>11601612.35</v>
       </c>
       <c r="Q22" s="9" t="n">
-        <v>283809889.14</v>
+        <v>283810892.72</v>
       </c>
       <c r="R22" s="10" t="n">
         <v>0.180964978836361</v>
@@ -1766,7 +1766,7 @@
         </is>
       </c>
       <c r="B23" s="5" t="n">
-        <v>1003048142.35</v>
+        <v>1003053368.32</v>
       </c>
       <c r="C23" s="6" t="n">
         <v>118302722.67</v>
@@ -1787,10 +1787,10 @@
         <v>9456461</v>
       </c>
       <c r="I23" s="7" t="n">
-        <v>1198204830.41</v>
+        <v>1198210056.38</v>
       </c>
       <c r="J23" s="8" t="n">
-        <v>222078381.47</v>
+        <v>222081575.1</v>
       </c>
       <c r="K23" s="9" t="n">
         <v>35142057.4</v>
@@ -1802,16 +1802,16 @@
         <v>577229.27</v>
       </c>
       <c r="N23" s="9" t="n">
-        <v>3890999.55</v>
+        <v>3891027.83</v>
       </c>
       <c r="O23" s="9" t="n">
-        <v>6335872.31</v>
+        <v>6335918.36</v>
       </c>
       <c r="P23" s="9" t="n">
         <v>3594255.85</v>
       </c>
       <c r="Q23" s="9" t="n">
-        <v>281009748.26</v>
+        <v>281013016.22</v>
       </c>
       <c r="R23" s="10" t="n">
         <v>0.316619068118602</v>
@@ -1824,7 +1824,7 @@
         </is>
       </c>
       <c r="B24" s="5" t="n">
-        <v>1362246646.22</v>
+        <v>1362253416.36</v>
       </c>
       <c r="C24" s="6" t="n">
         <v>146513108.49</v>
@@ -1845,10 +1845,10 @@
         <v>21014051</v>
       </c>
       <c r="I24" s="7" t="n">
-        <v>1634463401.34</v>
+        <v>1634470171.48</v>
       </c>
       <c r="J24" s="8" t="n">
-        <v>306752950.06</v>
+        <v>306754734.38</v>
       </c>
       <c r="K24" s="9" t="n">
         <v>43271898.85</v>
@@ -1860,16 +1860,16 @@
         <v>545961.96</v>
       </c>
       <c r="N24" s="9" t="n">
-        <v>6136465.49</v>
+        <v>6136468.41</v>
       </c>
       <c r="O24" s="9" t="n">
-        <v>10270554.21</v>
+        <v>10270559.1</v>
       </c>
       <c r="P24" s="9" t="n">
         <v>9618578.710000001</v>
       </c>
       <c r="Q24" s="9" t="n">
-        <v>388012101.25</v>
+        <v>388013893.39</v>
       </c>
       <c r="R24" s="10" t="n">
         <v>0.3069045894333504</v>
@@ -1882,7 +1882,7 @@
         </is>
       </c>
       <c r="B25" s="5" t="n">
-        <v>1156848829.83</v>
+        <v>1156855385.09</v>
       </c>
       <c r="C25" s="6" t="n">
         <v>144797057.56</v>
@@ -1903,10 +1903,10 @@
         <v>21174047</v>
       </c>
       <c r="I25" s="7" t="n">
-        <v>1409348797.48</v>
+        <v>1409355352.74</v>
       </c>
       <c r="J25" s="8" t="n">
-        <v>247783486.21</v>
+        <v>247785242.3</v>
       </c>
       <c r="K25" s="9" t="n">
         <v>45249277.15</v>
@@ -1918,16 +1918,16 @@
         <v>678289.72</v>
       </c>
       <c r="N25" s="9" t="n">
-        <v>3795191.26</v>
+        <v>3795194.18</v>
       </c>
       <c r="O25" s="9" t="n">
-        <v>9929275.09</v>
+        <v>9929282.720000001</v>
       </c>
       <c r="P25" s="9" t="n">
         <v>10104181.45</v>
       </c>
       <c r="Q25" s="9" t="n">
-        <v>325981177.34</v>
+        <v>325982943.97</v>
       </c>
       <c r="R25" s="10" t="n">
         <v>0.2790295913221863</v>
@@ -1940,7 +1940,7 @@
         </is>
       </c>
       <c r="B26" s="5" t="n">
-        <v>870234303.1799999</v>
+        <v>870241470.6900001</v>
       </c>
       <c r="C26" s="6" t="n">
         <v>97537800.47</v>
@@ -1961,10 +1961,10 @@
         <v>11503296</v>
       </c>
       <c r="I26" s="7" t="n">
-        <v>1039338515.55</v>
+        <v>1039345683.06</v>
       </c>
       <c r="J26" s="8" t="n">
-        <v>193417623.28</v>
+        <v>193419842.54</v>
       </c>
       <c r="K26" s="9" t="n">
         <v>31464287.45</v>
@@ -1976,16 +1976,16 @@
         <v>240533.84</v>
       </c>
       <c r="N26" s="9" t="n">
-        <v>3256064.62</v>
+        <v>3256071.89</v>
       </c>
       <c r="O26" s="9" t="n">
-        <v>5684208.02</v>
+        <v>5684220.72</v>
       </c>
       <c r="P26" s="9" t="n">
         <v>5132563.13</v>
       </c>
       <c r="Q26" s="9" t="n">
-        <v>245259707.55</v>
+        <v>245261946.78</v>
       </c>
       <c r="R26" s="10" t="n">
         <v>0.2509415863550032</v>
@@ -1998,7 +1998,7 @@
         </is>
       </c>
       <c r="B27" s="5" t="n">
-        <v>1002162415.6</v>
+        <v>1002174640.46</v>
       </c>
       <c r="C27" s="6" t="n">
         <v>122103455.85</v>
@@ -2019,10 +2019,10 @@
         <v>16332836</v>
       </c>
       <c r="I27" s="7" t="n">
-        <v>1209499823.56</v>
+        <v>1209512048.42</v>
       </c>
       <c r="J27" s="8" t="n">
-        <v>216979327.6</v>
+        <v>216983860.91</v>
       </c>
       <c r="K27" s="9" t="n">
         <v>38650744.49</v>
@@ -2034,16 +2034,16 @@
         <v>345067.73</v>
       </c>
       <c r="N27" s="9" t="n">
-        <v>2934170.27</v>
+        <v>2934188.6</v>
       </c>
       <c r="O27" s="9" t="n">
-        <v>6937774.34</v>
+        <v>6937817.69</v>
       </c>
       <c r="P27" s="9" t="n">
         <v>7469897.21</v>
       </c>
       <c r="Q27" s="9" t="n">
-        <v>280951677.29</v>
+        <v>280956272.28</v>
       </c>
       <c r="R27" s="10" t="n">
         <v>0.2836514946154119</v>
@@ -2056,7 +2056,7 @@
         </is>
       </c>
       <c r="B28" s="5" t="n">
-        <v>1105872460</v>
+        <v>1105897442.3</v>
       </c>
       <c r="C28" s="6" t="n">
         <v>146265225.05</v>
@@ -2077,10 +2077,10 @@
         <v>22808657</v>
       </c>
       <c r="I28" s="7" t="n">
-        <v>1351727359.65</v>
+        <v>1351752341.95</v>
       </c>
       <c r="J28" s="8" t="n">
-        <v>242452076.24</v>
+        <v>242461169.05</v>
       </c>
       <c r="K28" s="9" t="n">
         <v>47820263.66</v>
@@ -2092,16 +2092,16 @@
         <v>1170559.87</v>
       </c>
       <c r="N28" s="9" t="n">
-        <v>2693171.11</v>
+        <v>2693198.16</v>
       </c>
       <c r="O28" s="9" t="n">
-        <v>8763790.130000001</v>
+        <v>8763878.17</v>
       </c>
       <c r="P28" s="9" t="n">
         <v>10604681.86</v>
       </c>
       <c r="Q28" s="9" t="n">
-        <v>322765516.48</v>
+        <v>322774724.38</v>
       </c>
       <c r="R28" s="10" t="n">
         <v>0.2603327878455701</v>
@@ -2114,7 +2114,7 @@
         </is>
       </c>
       <c r="B29" s="5" t="n">
-        <v>932777126.6900001</v>
+        <v>932792254.42</v>
       </c>
       <c r="C29" s="6" t="n">
         <v>110832888.3</v>
@@ -2135,10 +2135,10 @@
         <v>22948569</v>
       </c>
       <c r="I29" s="7" t="n">
-        <v>1136724941.14</v>
+        <v>1136740068.87</v>
       </c>
       <c r="J29" s="8" t="n">
-        <v>196501497.97</v>
+        <v>196507493.81</v>
       </c>
       <c r="K29" s="9" t="n">
         <v>33469362.8</v>
@@ -2150,16 +2150,16 @@
         <v>3504492.28</v>
       </c>
       <c r="N29" s="9" t="n">
-        <v>2927838.11</v>
+        <v>2927867.9</v>
       </c>
       <c r="O29" s="9" t="n">
-        <v>6577645.92</v>
+        <v>6577712.84</v>
       </c>
       <c r="P29" s="9" t="n">
         <v>9864047.33</v>
       </c>
       <c r="Q29" s="9" t="n">
-        <v>259455323.36</v>
+        <v>259461415.9</v>
       </c>
       <c r="R29" s="10" t="n">
         <v>0.2711837542671093</v>
@@ -2172,7 +2172,7 @@
         </is>
       </c>
       <c r="B30" s="5" t="n">
-        <v>1161937950.78</v>
+        <v>1161965591.17</v>
       </c>
       <c r="C30" s="6" t="n">
         <v>97591814.65000001</v>
@@ -2193,10 +2193,10 @@
         <v>14181446</v>
       </c>
       <c r="I30" s="7" t="n">
-        <v>1354774434.85</v>
+        <v>1354802075.24</v>
       </c>
       <c r="J30" s="8" t="n">
-        <v>252320947.82</v>
+        <v>252334221.71</v>
       </c>
       <c r="K30" s="9" t="n">
         <v>30161405.65</v>
@@ -2208,16 +2208,16 @@
         <v>5547393.25</v>
       </c>
       <c r="N30" s="9" t="n">
-        <v>4229055.32</v>
+        <v>4229151.71</v>
       </c>
       <c r="O30" s="9" t="n">
-        <v>4541531.32</v>
+        <v>4541634.83</v>
       </c>
       <c r="P30" s="9" t="n">
         <v>5642292.92</v>
       </c>
       <c r="Q30" s="9" t="n">
-        <v>311933253.09</v>
+        <v>311946726.88</v>
       </c>
       <c r="R30" s="10" t="n">
         <v>0.3089090135319407</v>
@@ -2230,7 +2230,7 @@
         </is>
       </c>
       <c r="B31" s="5" t="n">
-        <v>1439894997.32</v>
+        <v>1439936873.53</v>
       </c>
       <c r="C31" s="6" t="n">
         <v>164444551.54</v>
@@ -2251,10 +2251,10 @@
         <v>25879178</v>
       </c>
       <c r="I31" s="7" t="n">
-        <v>1739951663.35</v>
+        <v>1739993539.56</v>
       </c>
       <c r="J31" s="8" t="n">
-        <v>284684023.21</v>
+        <v>284698738.36</v>
       </c>
       <c r="K31" s="9" t="n">
         <v>46737225.01</v>
@@ -2266,16 +2266,16 @@
         <v>10477277.08</v>
       </c>
       <c r="N31" s="9" t="n">
-        <v>4066960.53</v>
+        <v>4067023.69</v>
       </c>
       <c r="O31" s="9" t="n">
-        <v>5978325.02</v>
+        <v>5978417.86</v>
       </c>
       <c r="P31" s="9" t="n">
         <v>11977848.09</v>
       </c>
       <c r="Q31" s="9" t="n">
-        <v>375554497.62</v>
+        <v>375569368.77</v>
       </c>
       <c r="R31" s="10" t="n">
         <v>0.3202852257171364</v>
@@ -2288,7 +2288,7 @@
         </is>
       </c>
       <c r="B32" s="5" t="n">
-        <v>1319471126.18</v>
+        <v>1319619795.01</v>
       </c>
       <c r="C32" s="6" t="n">
         <v>152797571.95</v>
@@ -2309,10 +2309,10 @@
         <v>30594436</v>
       </c>
       <c r="I32" s="7" t="n">
-        <v>1579234210.3</v>
+        <v>1579382879.13</v>
       </c>
       <c r="J32" s="8" t="n">
-        <v>283287864.82</v>
+        <v>283347224.81</v>
       </c>
       <c r="K32" s="9" t="n">
         <v>45961937.88</v>
@@ -2324,16 +2324,16 @@
         <v>1721674.99</v>
       </c>
       <c r="N32" s="9" t="n">
-        <v>3050704.66</v>
+        <v>3050921.86</v>
       </c>
       <c r="O32" s="9" t="n">
-        <v>7437769.93</v>
+        <v>7438299.47</v>
       </c>
       <c r="P32" s="9" t="n">
         <v>14143642.2</v>
       </c>
       <c r="Q32" s="9" t="n">
-        <v>363527703.93</v>
+        <v>363587810.66</v>
       </c>
       <c r="R32" s="10" t="n">
         <v>0.3068596818867773</v>
@@ -2346,7 +2346,7 @@
         </is>
       </c>
       <c r="B33" s="5" t="n">
-        <v>1096650095.4</v>
+        <v>1096905074.29</v>
       </c>
       <c r="C33" s="6" t="n">
         <v>112904481.21</v>
@@ -2367,10 +2367,10 @@
         <v>10653135</v>
       </c>
       <c r="I33" s="7" t="n">
-        <v>1282691121.51</v>
+        <v>1282946100.4</v>
       </c>
       <c r="J33" s="8" t="n">
-        <v>243300304.72</v>
+        <v>243398809.77</v>
       </c>
       <c r="K33" s="9" t="n">
         <v>36710222.03</v>
@@ -2382,16 +2382,16 @@
         <v>7580.34</v>
       </c>
       <c r="N33" s="9" t="n">
-        <v>1660372.72</v>
+        <v>1660590.55</v>
       </c>
       <c r="O33" s="9" t="n">
-        <v>7200948.89</v>
+        <v>7201893.64</v>
       </c>
       <c r="P33" s="9" t="n">
         <v>4972134.8</v>
       </c>
       <c r="Q33" s="9" t="n">
-        <v>302016517.86</v>
+        <v>302116185.49</v>
       </c>
       <c r="R33" s="10" t="n">
         <v>0.2945849325840212</v>
@@ -2404,7 +2404,7 @@
         </is>
       </c>
       <c r="B34" s="5" t="n">
-        <v>1141713194.51</v>
+        <v>1141995936.6</v>
       </c>
       <c r="C34" s="6" t="n">
         <v>111143033.33</v>
@@ -2425,10 +2425,10 @@
         <v>17975675</v>
       </c>
       <c r="I34" s="7" t="n">
-        <v>1365604308.46</v>
+        <v>1365887050.55</v>
       </c>
       <c r="J34" s="8" t="n">
-        <v>239505889.8</v>
+        <v>239622450.68</v>
       </c>
       <c r="K34" s="9" t="n">
         <v>33583851.03</v>
@@ -2440,16 +2440,16 @@
         <v>7000711.88</v>
       </c>
       <c r="N34" s="9" t="n">
-        <v>1298241.07</v>
+        <v>1298472.6</v>
       </c>
       <c r="O34" s="9" t="n">
-        <v>9232363.02</v>
+        <v>9234009.52</v>
       </c>
       <c r="P34" s="9" t="n">
         <v>8253527.4</v>
       </c>
       <c r="Q34" s="9" t="n">
-        <v>307296868.64</v>
+        <v>307415307.54</v>
       </c>
       <c r="R34" s="10" t="n">
         <v>0.3414174721986673</v>
@@ -2462,7 +2462,7 @@
         </is>
       </c>
       <c r="B35" s="5" t="n">
-        <v>1192398704.86</v>
+        <v>1192713713.87</v>
       </c>
       <c r="C35" s="6" t="n">
         <v>132482292.68</v>
@@ -2483,10 +2483,10 @@
         <v>24222748</v>
       </c>
       <c r="I35" s="7" t="n">
-        <v>1436055711.53</v>
+        <v>1436370720.54</v>
       </c>
       <c r="J35" s="8" t="n">
-        <v>253455797.87</v>
+        <v>253585262.84</v>
       </c>
       <c r="K35" s="9" t="n">
         <v>39009606.34</v>
@@ -2498,16 +2498,16 @@
         <v>7686788.4</v>
       </c>
       <c r="N35" s="9" t="n">
-        <v>2144828.4</v>
+        <v>2145215.4</v>
       </c>
       <c r="O35" s="9" t="n">
-        <v>6743602.9</v>
+        <v>6744819.69</v>
       </c>
       <c r="P35" s="9" t="n">
         <v>11819801.92</v>
       </c>
       <c r="Q35" s="9" t="n">
-        <v>327808631.37</v>
+        <v>327939700.13</v>
       </c>
       <c r="R35" s="10" t="n">
         <v>0.3444918139984984</v>
@@ -2520,7 +2520,7 @@
         </is>
       </c>
       <c r="B36" s="5" t="n">
-        <v>1226269672.23</v>
+        <v>1226786729.91</v>
       </c>
       <c r="C36" s="6" t="n">
         <v>147816672.25</v>
@@ -2541,10 +2541,10 @@
         <v>27056266</v>
       </c>
       <c r="I36" s="7" t="n">
-        <v>1493609963.1</v>
+        <v>1494127020.78</v>
       </c>
       <c r="J36" s="8" t="n">
-        <v>272681676.9</v>
+        <v>272903711.42</v>
       </c>
       <c r="K36" s="9" t="n">
         <v>47162206.4</v>
@@ -2556,16 +2556,16 @@
         <v>8799940.630000001</v>
       </c>
       <c r="N36" s="9" t="n">
-        <v>2511016.2</v>
+        <v>2511710.21</v>
       </c>
       <c r="O36" s="9" t="n">
-        <v>7245924.46</v>
+        <v>7247927.12</v>
       </c>
       <c r="P36" s="9" t="n">
         <v>13258351.53</v>
       </c>
       <c r="Q36" s="9" t="n">
-        <v>360920702.24</v>
+        <v>361145433.43</v>
       </c>
       <c r="R36" s="10" t="n">
         <v>0.3000842795719814</v>
@@ -2578,7 +2578,7 @@
         </is>
       </c>
       <c r="B37" s="5" t="n">
-        <v>1172274619.91</v>
+        <v>1324835906.41</v>
       </c>
       <c r="C37" s="6" t="n">
         <v>161563894</v>
@@ -2599,10 +2599,10 @@
         <v>12713214</v>
       </c>
       <c r="I37" s="7" t="n">
-        <v>1446594764.66</v>
+        <v>1599156051.16</v>
       </c>
       <c r="J37" s="8" t="n">
-        <v>244007566.85</v>
+        <v>276866413.12</v>
       </c>
       <c r="K37" s="9" t="n">
         <v>49969403.31</v>
@@ -2614,16 +2614,16 @@
         <v>7004156.33</v>
       </c>
       <c r="N37" s="9" t="n">
-        <v>2343656.88</v>
+        <v>2332415.96</v>
       </c>
       <c r="O37" s="9" t="n">
-        <v>8215141.66</v>
+        <v>8175739.23</v>
       </c>
       <c r="P37" s="9" t="n">
         <v>5644731.29</v>
       </c>
       <c r="Q37" s="9" t="n">
-        <v>327557272.18</v>
+        <v>360365475.1</v>
       </c>
       <c r="R37" s="10" t="n">
         <v>0.3158320960096582</v>
@@ -2635,7 +2635,9 @@
           <t>2026-09-05</t>
         </is>
       </c>
-      <c r="B38" s="5" t="n"/>
+      <c r="B38" s="5" t="n">
+        <v>1803304137.56</v>
+      </c>
       <c r="C38" s="6" t="n">
         <v>172439695.17</v>
       </c>
@@ -2655,9 +2657,11 @@
         <v>20531449</v>
       </c>
       <c r="I38" s="7" t="n">
-        <v>344063062.06</v>
-      </c>
-      <c r="J38" s="8" t="n"/>
+        <v>2147367199.62</v>
+      </c>
+      <c r="J38" s="8" t="n">
+        <v>365996657.83</v>
+      </c>
       <c r="K38" s="9" t="n">
         <v>46814559.69</v>
       </c>
@@ -2668,16 +2672,16 @@
         <v>15883449.41</v>
       </c>
       <c r="N38" s="9" t="n">
-        <v>5461948.41</v>
+        <v>3885058.95</v>
       </c>
       <c r="O38" s="9" t="n">
-        <v>9263993.560000001</v>
+        <v>6589436.3</v>
       </c>
       <c r="P38" s="9" t="n">
         <v>9731632.92</v>
       </c>
       <c r="Q38" s="9" t="n">
-        <v>105178709.74</v>
+        <v>466923920.86</v>
       </c>
       <c r="R38" s="10" t="n">
         <v>0.3730201375328469</v>
@@ -2693,12 +2697,8 @@
       <c r="C39" s="6" t="n">
         <v>131412975.25</v>
       </c>
-      <c r="D39" s="6" t="n">
-        <v>32056055.97</v>
-      </c>
-      <c r="E39" s="6" t="n">
-        <v>35925674</v>
-      </c>
+      <c r="D39" s="6" t="n"/>
+      <c r="E39" s="6" t="n"/>
       <c r="F39" s="6" t="n">
         <v>21673332.38</v>
       </c>
@@ -2709,36 +2709,70 @@
         <v>33293997</v>
       </c>
       <c r="I39" s="7" t="n">
-        <v>286769786.6</v>
+        <v>218788056.63</v>
       </c>
       <c r="J39" s="8" t="n"/>
       <c r="K39" s="9" t="n">
         <v>38038258.86</v>
       </c>
-      <c r="L39" s="9" t="n">
-        <v>13010644.31</v>
-      </c>
-      <c r="M39" s="9" t="n">
-        <v>11501420.69</v>
-      </c>
+      <c r="L39" s="9" t="n"/>
+      <c r="M39" s="9" t="n"/>
       <c r="N39" s="9" t="n">
-        <v>7323631.12</v>
+        <v>7120937.7</v>
       </c>
       <c r="O39" s="9" t="n">
-        <v>10950896.56</v>
+        <v>10647812.66</v>
       </c>
       <c r="P39" s="9" t="n">
         <v>16077465.82</v>
       </c>
       <c r="Q39" s="9" t="n">
-        <v>96902317.34999999</v>
+        <v>71884475.04000001</v>
       </c>
       <c r="R39" s="10" t="n">
-        <v>0.3654745795652588</v>
+        <v>0.3594880079566298</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-07</t>
+        </is>
+      </c>
+      <c r="B40" s="5" t="n"/>
+      <c r="C40" s="6" t="n"/>
+      <c r="D40" s="6" t="n"/>
+      <c r="E40" s="6" t="n"/>
+      <c r="F40" s="6" t="n"/>
+      <c r="G40" s="6" t="n">
+        <v>19529310</v>
+      </c>
+      <c r="H40" s="6" t="n">
+        <v>36648697</v>
+      </c>
+      <c r="I40" s="7" t="n">
+        <v>56178007</v>
+      </c>
+      <c r="J40" s="8" t="n"/>
+      <c r="K40" s="9" t="n"/>
+      <c r="L40" s="9" t="n"/>
+      <c r="M40" s="9" t="n"/>
+      <c r="N40" s="9" t="n"/>
+      <c r="O40" s="9" t="n">
+        <v>9844830.470000001</v>
+      </c>
+      <c r="P40" s="9" t="n">
+        <v>18474805.77</v>
+      </c>
+      <c r="Q40" s="9" t="n">
+        <v>28319636.24</v>
+      </c>
+      <c r="R40" s="10" t="n">
+        <v>0.3616</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A2:R39"/>
+  <autoFilter ref="A2:R40"/>
   <mergeCells count="3">
     <mergeCell ref="R1"/>
     <mergeCell ref="B1:I1"/>
@@ -2754,7 +2788,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q39"/>
+  <dimension ref="A1:Q40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -4740,7 +4774,7 @@
         </is>
       </c>
       <c r="B37" s="5" t="n">
-        <v>1523154175.75</v>
+        <v>1721050019.04</v>
       </c>
       <c r="C37" s="6" t="n">
         <v>162404936.11</v>
@@ -4761,10 +4795,10 @@
         <v>14064111</v>
       </c>
       <c r="I37" s="7" t="n">
-        <v>1801932379.61</v>
+        <v>1999828222.9</v>
       </c>
       <c r="J37" s="8" t="n">
-        <v>422827599.19</v>
+        <v>477763485.29</v>
       </c>
       <c r="K37" s="9" t="n">
         <v>50100849.41</v>
@@ -4776,16 +4810,16 @@
         <v>7004156.33</v>
       </c>
       <c r="N37" s="9" t="n">
-        <v>2931559.34</v>
+        <v>2925644.45</v>
       </c>
       <c r="O37" s="9" t="n">
-        <v>10917738.06</v>
+        <v>10895709.78</v>
       </c>
       <c r="P37" s="9" t="n">
         <v>6213562.76</v>
       </c>
       <c r="Q37" s="9" t="n">
-        <v>510368080.94</v>
+        <v>565276023.87</v>
       </c>
     </row>
     <row r="38">
@@ -4794,7 +4828,9 @@
           <t>2026-09-05</t>
         </is>
       </c>
-      <c r="B38" s="5" t="n"/>
+      <c r="B38" s="5" t="n">
+        <v>2342612096.54</v>
+      </c>
       <c r="C38" s="6" t="n">
         <v>173014888.85</v>
       </c>
@@ -4814,9 +4850,11 @@
         <v>21111711</v>
       </c>
       <c r="I38" s="7" t="n">
-        <v>346849792.74</v>
-      </c>
-      <c r="J38" s="8" t="n"/>
+        <v>2689461889.28</v>
+      </c>
+      <c r="J38" s="8" t="n">
+        <v>650309118</v>
+      </c>
       <c r="K38" s="9" t="n">
         <v>46914612.74</v>
       </c>
@@ -4827,16 +4865,16 @@
         <v>15883449.41</v>
       </c>
       <c r="N38" s="9" t="n">
-        <v>5459538.21</v>
+        <v>5016169.45</v>
       </c>
       <c r="O38" s="9" t="n">
-        <v>9758359.859999999</v>
+        <v>8965884.060000001</v>
       </c>
       <c r="P38" s="9" t="n">
         <v>9944728.02</v>
       </c>
       <c r="Q38" s="9" t="n">
-        <v>105983813.98</v>
+        <v>755057087.4299999</v>
       </c>
     </row>
     <row r="39">
@@ -4849,12 +4887,8 @@
       <c r="C39" s="6" t="n">
         <v>132077170.89</v>
       </c>
-      <c r="D39" s="6" t="n">
-        <v>32056055.97</v>
-      </c>
-      <c r="E39" s="6" t="n">
-        <v>35925674</v>
-      </c>
+      <c r="D39" s="6" t="n"/>
+      <c r="E39" s="6" t="n"/>
       <c r="F39" s="6" t="n">
         <v>21673332.38</v>
       </c>
@@ -4865,33 +4899,64 @@
         <v>33781884</v>
       </c>
       <c r="I39" s="7" t="n">
-        <v>290377632.24</v>
+        <v>222395902.27</v>
       </c>
       <c r="J39" s="8" t="n"/>
       <c r="K39" s="9" t="n">
         <v>38188228.54</v>
       </c>
-      <c r="L39" s="9" t="n">
-        <v>13010644.31</v>
-      </c>
-      <c r="M39" s="9" t="n">
-        <v>11501420.69</v>
-      </c>
+      <c r="L39" s="9" t="n"/>
+      <c r="M39" s="9" t="n"/>
       <c r="N39" s="9" t="n">
-        <v>7315628</v>
+        <v>7111062.23</v>
       </c>
       <c r="O39" s="9" t="n">
-        <v>11767849.17</v>
+        <v>11438786.63</v>
       </c>
       <c r="P39" s="9" t="n">
         <v>16230447.81</v>
       </c>
       <c r="Q39" s="9" t="n">
-        <v>98014218.51000001</v>
+        <v>72968525.2</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-07</t>
+        </is>
+      </c>
+      <c r="B40" s="5" t="n"/>
+      <c r="C40" s="6" t="n"/>
+      <c r="D40" s="6" t="n"/>
+      <c r="E40" s="6" t="n"/>
+      <c r="F40" s="6" t="n"/>
+      <c r="G40" s="6" t="n">
+        <v>21831205</v>
+      </c>
+      <c r="H40" s="6" t="n">
+        <v>37074913</v>
+      </c>
+      <c r="I40" s="7" t="n">
+        <v>58906118</v>
+      </c>
+      <c r="J40" s="8" t="n"/>
+      <c r="K40" s="9" t="n"/>
+      <c r="L40" s="9" t="n"/>
+      <c r="M40" s="9" t="n"/>
+      <c r="N40" s="9" t="n"/>
+      <c r="O40" s="9" t="n">
+        <v>10966998.92</v>
+      </c>
+      <c r="P40" s="9" t="n">
+        <v>18624740.64</v>
+      </c>
+      <c r="Q40" s="9" t="n">
+        <v>29591739.56</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A2:Q39"/>
+  <autoFilter ref="A2:Q40"/>
   <mergeCells count="2">
     <mergeCell ref="B1:I1"/>
     <mergeCell ref="J1:Q1"/>
@@ -4906,7 +4971,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M41"/>
+  <dimension ref="A1:M42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -6134,7 +6199,7 @@
         <v>9008514</v>
       </c>
       <c r="H29" s="11" t="n">
-        <v>0.6143999999999999</v>
+        <v>0.6143</v>
       </c>
       <c r="I29" s="11" t="n">
         <v>0.3433</v>
@@ -6306,7 +6371,7 @@
         <v>9774024</v>
       </c>
       <c r="H33" s="11" t="n">
-        <v>0.6148</v>
+        <v>0.6146</v>
       </c>
       <c r="I33" s="11" t="n">
         <v>0.4301</v>
@@ -6349,7 +6414,7 @@
         <v>12995978</v>
       </c>
       <c r="H34" s="11" t="n">
-        <v>0.6411</v>
+        <v>0.6409999999999999</v>
       </c>
       <c r="I34" s="11" t="n">
         <v>0.474</v>
@@ -6392,7 +6457,7 @@
         <v>10158090</v>
       </c>
       <c r="H35" s="11" t="n">
-        <v>0.6381</v>
+        <v>0.6379</v>
       </c>
       <c r="I35" s="11" t="n">
         <v>0.4234000000000001</v>
@@ -6435,7 +6500,7 @@
         <v>8471978</v>
       </c>
       <c r="H36" s="11" t="n">
-        <v>0.6048</v>
+        <v>0.6045</v>
       </c>
       <c r="I36" s="11" t="n">
         <v>0.3584000000000001</v>
@@ -6460,7 +6525,7 @@
         </is>
       </c>
       <c r="B37" s="6" t="n">
-        <v>733490124.87</v>
+        <v>828788847.17</v>
       </c>
       <c r="C37" s="6" t="n">
         <v>12490106.43</v>
@@ -6478,7 +6543,7 @@
         <v>11868618</v>
       </c>
       <c r="H37" s="11" t="n">
-        <v>0.6257</v>
+        <v>0.6256</v>
       </c>
       <c r="I37" s="11" t="n">
         <v>0.3806</v>
@@ -6502,7 +6567,9 @@
           <t>2026-09-05</t>
         </is>
       </c>
-      <c r="B38" s="6" t="n"/>
+      <c r="B38" s="6" t="n">
+        <v>1128108281.21</v>
+      </c>
       <c r="C38" s="6" t="n">
         <v>18169819.03</v>
       </c>
@@ -6518,7 +6585,9 @@
       <c r="G38" s="6" t="n">
         <v>10824093</v>
       </c>
-      <c r="H38" s="11" t="n"/>
+      <c r="H38" s="11" t="n">
+        <v>0.6256</v>
+      </c>
       <c r="I38" s="11" t="n">
         <v>0.3624</v>
       </c>
@@ -6542,12 +6611,8 @@
         </is>
       </c>
       <c r="B39" s="6" t="n"/>
-      <c r="C39" s="6" t="n">
-        <v>10625376.42</v>
-      </c>
-      <c r="D39" s="6" t="n">
-        <v>15329162</v>
-      </c>
+      <c r="C39" s="6" t="n"/>
+      <c r="D39" s="6" t="n"/>
       <c r="E39" s="6" t="n">
         <v>40590069.68</v>
       </c>
@@ -6558,12 +6623,8 @@
         <v>12319196</v>
       </c>
       <c r="H39" s="11" t="n"/>
-      <c r="I39" s="11" t="n">
-        <v>0.3315</v>
-      </c>
-      <c r="J39" s="11" t="n">
-        <v>0.4267</v>
-      </c>
+      <c r="I39" s="11" t="n"/>
+      <c r="J39" s="11" t="n"/>
       <c r="K39" s="11" t="n">
         <v>0.3089</v>
       </c>
@@ -6574,15 +6635,38 @@
         <v>0.3801</v>
       </c>
     </row>
-    <row r="41">
-      <c r="A41" s="12" t="inlineStr">
+    <row r="40">
+      <c r="A40" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-07</t>
+        </is>
+      </c>
+      <c r="B40" s="6" t="n"/>
+      <c r="C40" s="6" t="n"/>
+      <c r="D40" s="6" t="n"/>
+      <c r="E40" s="6" t="n"/>
+      <c r="F40" s="6" t="n"/>
+      <c r="G40" s="6" t="n">
+        <v>7061846</v>
+      </c>
+      <c r="H40" s="11" t="n"/>
+      <c r="I40" s="11" t="n"/>
+      <c r="J40" s="11" t="n"/>
+      <c r="K40" s="11" t="n"/>
+      <c r="L40" s="11" t="n"/>
+      <c r="M40" s="11" t="n">
+        <v>0.3616</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="12" t="inlineStr">
         <is>
           <t>Combo % = parlay volume / that venue's sports book. Kalshi's parlay is its KXMVE multi-event engine (leg-checked ~100% sports legs despite the 'cross-category' name), from a ~3M-trade sample scaled to the daily total; ~62% of Kalshi's sports book by contracts, ~18% by $ (parlay legs are many and cheap). Not folded into the Sports tab's blended Combo % (sample-based, moves less day to day). Rothera runs no on-exchange parlay product.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A2:M39"/>
+  <autoFilter ref="A2:M40"/>
   <mergeCells count="2">
     <mergeCell ref="H1:M1"/>
     <mergeCell ref="B1:G1"/>
@@ -6613,7 +6697,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Generated 2026-09-07. Full detail: VOLUME_METHODOLOGY.md</t>
+          <t>Generated 2026-09-08. Full detail: VOLUME_METHODOLOGY.md</t>
         </is>
       </c>
     </row>

</xml_diff>